<commit_message>
0705 test: 45 rows, 42 exact + 3 new, K sum=1084, all verified
</commit_message>
<xml_diff>
--- a/2607.xlsx
+++ b/2607.xlsx
@@ -8,22 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\me\致知收益\2025\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CE2D43D-1EB0-4B89-A7D3-BC4E699056F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D553FA4-6BC2-424F-8C39-37B99455D0B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="0701" sheetId="1" r:id="rId1"/>
     <sheet name="0702" sheetId="2" r:id="rId2"/>
     <sheet name="0703" sheetId="3" r:id="rId3"/>
     <sheet name="0704" sheetId="4" r:id="rId4"/>
+    <sheet name="0705" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="181029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="600" uniqueCount="104">
   <si>
     <t>内容</t>
   </si>
@@ -324,14 +325,26 @@
   <si>
     <t>合计</t>
   </si>
+  <si>
+    <t>L0705</t>
+  </si>
+  <si>
+    <t>对比写程序完成与手动完成，2天与2分钟，到底哪一种方式更适合？知乎电脑版“收益分析”项，默...</t>
+  </si>
+  <si>
+    <t>6 月以来金星高悬夜空，它达到一年中地平高度最高点的天文原因是什么？</t>
+  </si>
+  <si>
+    <t>如何知道你的狗狗生活的很快乐？</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="178" formatCode="0.00_ "/>
-    <numFmt numFmtId="179" formatCode="0_ "/>
+    <numFmt numFmtId="176" formatCode="0.00_ "/>
+    <numFmt numFmtId="177" formatCode="0_ "/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -384,16 +397,16 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1">
+    <xf numFmtId="177" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -7245,11 +7258,11 @@
         <v>175</v>
       </c>
       <c r="H2">
-        <f>ROUND(E2/D2,2)</f>
+        <f t="shared" ref="H2:H48" si="0">ROUND(E2/D2,2)</f>
         <v>0.08</v>
       </c>
       <c r="I2">
-        <f>ROUND(G2/F2,2)</f>
+        <f t="shared" ref="I2:I48" si="1">ROUND(G2/F2,2)</f>
         <v>0.08</v>
       </c>
       <c r="J2">
@@ -7261,7 +7274,7 @@
         <v>44</v>
       </c>
       <c r="L2">
-        <f>IFERROR(ROUND(K2/J2,2),)</f>
+        <f t="shared" ref="L2:L48" si="2">IFERROR(ROUND(K2/J2,2),)</f>
         <v>0.13</v>
       </c>
     </row>
@@ -7288,11 +7301,11 @@
         <v>991</v>
       </c>
       <c r="H3">
-        <f>ROUND(E3/D3,2)</f>
+        <f t="shared" si="0"/>
         <v>1.91</v>
       </c>
       <c r="I3">
-        <f>ROUND(G3/F3,2)</f>
+        <f t="shared" si="1"/>
         <v>1.91</v>
       </c>
       <c r="J3">
@@ -7304,7 +7317,7 @@
         <v>258</v>
       </c>
       <c r="L3">
-        <f>IFERROR(ROUND(K3/J3,2),)</f>
+        <f t="shared" si="2"/>
         <v>0.81</v>
       </c>
     </row>
@@ -7331,11 +7344,11 @@
         <v>241</v>
       </c>
       <c r="H4">
-        <f>ROUND(E4/D4,2)</f>
+        <f t="shared" si="0"/>
         <v>0.45</v>
       </c>
       <c r="I4">
-        <f>ROUND(G4/F4,2)</f>
+        <f t="shared" si="1"/>
         <v>0.45</v>
       </c>
       <c r="J4">
@@ -7347,7 +7360,7 @@
         <v>29</v>
       </c>
       <c r="L4">
-        <f>IFERROR(ROUND(K4/J4,2),)</f>
+        <f t="shared" si="2"/>
         <v>0.45</v>
       </c>
     </row>
@@ -7374,11 +7387,11 @@
         <v>317</v>
       </c>
       <c r="H5">
-        <f>ROUND(E5/D5,2)</f>
+        <f t="shared" si="0"/>
         <v>2.13</v>
       </c>
       <c r="I5">
-        <f>ROUND(G5/F5,2)</f>
+        <f t="shared" si="1"/>
         <v>2.13</v>
       </c>
       <c r="J5">
@@ -7390,7 +7403,7 @@
         <v>7</v>
       </c>
       <c r="L5">
-        <f>IFERROR(ROUND(K5/J5,2),)</f>
+        <f t="shared" si="2"/>
         <v>0.37</v>
       </c>
     </row>
@@ -7417,11 +7430,11 @@
         <v>655</v>
       </c>
       <c r="H6">
-        <f>ROUND(E6/D6,2)</f>
+        <f t="shared" si="0"/>
         <v>8.19</v>
       </c>
       <c r="I6">
-        <f>ROUND(G6/F6,2)</f>
+        <f t="shared" si="1"/>
         <v>8.19</v>
       </c>
       <c r="J6">
@@ -7433,7 +7446,7 @@
         <v>17</v>
       </c>
       <c r="L6">
-        <f>IFERROR(ROUND(K6/J6,2),)</f>
+        <f t="shared" si="2"/>
         <v>3.4</v>
       </c>
     </row>
@@ -7460,11 +7473,11 @@
         <v>114</v>
       </c>
       <c r="H7">
-        <f>ROUND(E7/D7,2)</f>
+        <f t="shared" si="0"/>
         <v>0.14000000000000001</v>
       </c>
       <c r="I7">
-        <f>ROUND(G7/F7,2)</f>
+        <f t="shared" si="1"/>
         <v>0.14000000000000001</v>
       </c>
       <c r="J7">
@@ -7476,7 +7489,7 @@
         <v>0</v>
       </c>
       <c r="L7">
-        <f>IFERROR(ROUND(K7/J7,2),)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -7503,11 +7516,11 @@
         <v>918</v>
       </c>
       <c r="H8">
-        <f>ROUND(E8/D8,2)</f>
+        <f t="shared" si="0"/>
         <v>8.83</v>
       </c>
       <c r="I8">
-        <f>ROUND(G8/F8,2)</f>
+        <f t="shared" si="1"/>
         <v>8.83</v>
       </c>
       <c r="J8">
@@ -7519,7 +7532,7 @@
         <v>51</v>
       </c>
       <c r="L8">
-        <f>IFERROR(ROUND(K8/J8,2),)</f>
+        <f t="shared" si="2"/>
         <v>6.38</v>
       </c>
       <c r="M8" t="s">
@@ -7549,11 +7562,11 @@
         <v>205</v>
       </c>
       <c r="H9">
-        <f>ROUND(E9/D9,2)</f>
+        <f t="shared" si="0"/>
         <v>0.41</v>
       </c>
       <c r="I9">
-        <f>ROUND(G9/F9,2)</f>
+        <f t="shared" si="1"/>
         <v>0.41</v>
       </c>
       <c r="J9">
@@ -7565,7 +7578,7 @@
         <v>0</v>
       </c>
       <c r="L9">
-        <f>IFERROR(ROUND(K9/J9,2),)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -7592,11 +7605,11 @@
         <v>310</v>
       </c>
       <c r="H10">
-        <f>ROUND(E10/D10,2)</f>
+        <f t="shared" si="0"/>
         <v>0.73</v>
       </c>
       <c r="I10">
-        <f>ROUND(G10/F10,2)</f>
+        <f t="shared" si="1"/>
         <v>0.73</v>
       </c>
       <c r="J10">
@@ -7608,7 +7621,7 @@
         <v>0</v>
       </c>
       <c r="L10">
-        <f>IFERROR(ROUND(K10/J10,2),)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -7635,11 +7648,11 @@
         <v>967</v>
       </c>
       <c r="H11">
-        <f>ROUND(E11/D11,2)</f>
+        <f t="shared" si="0"/>
         <v>2.99</v>
       </c>
       <c r="I11">
-        <f>ROUND(G11/F11,2)</f>
+        <f t="shared" si="1"/>
         <v>2.99</v>
       </c>
       <c r="J11">
@@ -7651,7 +7664,7 @@
         <v>0</v>
       </c>
       <c r="L11">
-        <f>IFERROR(ROUND(K11/J11,2),)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -7678,11 +7691,11 @@
         <v>543</v>
       </c>
       <c r="H12">
-        <f>ROUND(E12/D12,2)</f>
+        <f t="shared" si="0"/>
         <v>3.42</v>
       </c>
       <c r="I12">
-        <f>ROUND(G12/F12,2)</f>
+        <f t="shared" si="1"/>
         <v>3.42</v>
       </c>
       <c r="J12">
@@ -7694,7 +7707,7 @@
         <v>51</v>
       </c>
       <c r="L12">
-        <f>IFERROR(ROUND(K12/J12,2),)</f>
+        <f t="shared" si="2"/>
         <v>3.92</v>
       </c>
     </row>
@@ -7721,11 +7734,11 @@
         <v>430</v>
       </c>
       <c r="H13">
-        <f>ROUND(E13/D13,2)</f>
+        <f t="shared" si="0"/>
         <v>3.31</v>
       </c>
       <c r="I13">
-        <f>ROUND(G13/F13,2)</f>
+        <f t="shared" si="1"/>
         <v>3.58</v>
       </c>
       <c r="J13">
@@ -7737,7 +7750,7 @@
         <v>0</v>
       </c>
       <c r="L13">
-        <f>IFERROR(ROUND(K13/J13,2),)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -7764,11 +7777,11 @@
         <v>198</v>
       </c>
       <c r="H14">
-        <f>ROUND(E14/D14,2)</f>
+        <f t="shared" si="0"/>
         <v>0.37</v>
       </c>
       <c r="I14">
-        <f>ROUND(G14/F14,2)</f>
+        <f t="shared" si="1"/>
         <v>0.33</v>
       </c>
       <c r="J14">
@@ -7780,7 +7793,7 @@
         <v>0</v>
       </c>
       <c r="L14">
-        <f>IFERROR(ROUND(K14/J14,2),)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -7807,11 +7820,11 @@
         <v>1437</v>
       </c>
       <c r="H15">
-        <f>ROUND(E15/D15,2)</f>
+        <f t="shared" si="0"/>
         <v>6.15</v>
       </c>
       <c r="I15">
-        <f>ROUND(G15/F15,2)</f>
+        <f t="shared" si="1"/>
         <v>6.91</v>
       </c>
       <c r="J15">
@@ -7823,7 +7836,7 @@
         <v>0</v>
       </c>
       <c r="L15">
-        <f>IFERROR(ROUND(K15/J15,2),)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -7850,11 +7863,11 @@
         <v>650</v>
       </c>
       <c r="H16">
-        <f>ROUND(E16/D16,2)</f>
+        <f t="shared" si="0"/>
         <v>5.52</v>
       </c>
       <c r="I16">
-        <f>ROUND(G16/F16,2)</f>
+        <f t="shared" si="1"/>
         <v>5.33</v>
       </c>
       <c r="J16">
@@ -7866,7 +7879,7 @@
         <v>0</v>
       </c>
       <c r="L16">
-        <f>IFERROR(ROUND(K16/J16,2),)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M16" t="s">
@@ -7899,11 +7912,11 @@
         <v>281</v>
       </c>
       <c r="H17">
-        <f>ROUND(E17/D17,2)</f>
+        <f t="shared" si="0"/>
         <v>0.1</v>
       </c>
       <c r="I17">
-        <f>ROUND(G17/F17,2)</f>
+        <f t="shared" si="1"/>
         <v>0.3</v>
       </c>
       <c r="J17">
@@ -7915,7 +7928,7 @@
         <v>0</v>
       </c>
       <c r="L17">
-        <f>IFERROR(ROUND(K17/J17,2),)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -7942,11 +7955,11 @@
         <v>1365</v>
       </c>
       <c r="H18">
-        <f>ROUND(E18/D18,2)</f>
+        <f t="shared" si="0"/>
         <v>5.66</v>
       </c>
       <c r="I18">
-        <f>ROUND(G18/F18,2)</f>
+        <f t="shared" si="1"/>
         <v>7</v>
       </c>
       <c r="J18">
@@ -7958,7 +7971,7 @@
         <v>69</v>
       </c>
       <c r="L18">
-        <f>IFERROR(ROUND(K18/J18,2),)</f>
+        <f t="shared" si="2"/>
         <v>9.86</v>
       </c>
       <c r="M18" t="s">
@@ -7988,11 +8001,11 @@
         <v>730</v>
       </c>
       <c r="H19">
-        <f>ROUND(E19/D19,2)</f>
+        <f t="shared" si="0"/>
         <v>5.31</v>
       </c>
       <c r="I19">
-        <f>ROUND(G19/F19,2)</f>
+        <f t="shared" si="1"/>
         <v>4.8</v>
       </c>
       <c r="J19">
@@ -8004,7 +8017,7 @@
         <v>0</v>
       </c>
       <c r="L19">
-        <f>IFERROR(ROUND(K19/J19,2),)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M19" t="s">
@@ -8037,11 +8050,11 @@
         <v>1024</v>
       </c>
       <c r="H20">
-        <f>ROUND(E20/D20,2)</f>
+        <f t="shared" si="0"/>
         <v>11.45</v>
       </c>
       <c r="I20">
-        <f>ROUND(G20/F20,2)</f>
+        <f t="shared" si="1"/>
         <v>6.65</v>
       </c>
       <c r="J20">
@@ -8053,7 +8066,7 @@
         <v>0</v>
       </c>
       <c r="L20">
-        <f>IFERROR(ROUND(K20/J20,2),)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M20" t="s">
@@ -8086,11 +8099,11 @@
         <v>114</v>
       </c>
       <c r="H21">
-        <f>ROUND(E21/D21,2)</f>
+        <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
       <c r="I21">
-        <f>ROUND(G21/F21,2)</f>
+        <f t="shared" si="1"/>
         <v>0.77</v>
       </c>
       <c r="J21">
@@ -8102,7 +8115,7 @@
         <v>0</v>
       </c>
       <c r="L21">
-        <f>IFERROR(ROUND(K21/J21,2),)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -8129,11 +8142,11 @@
         <v>1668</v>
       </c>
       <c r="H22">
-        <f>ROUND(E22/D22,2)</f>
+        <f t="shared" si="0"/>
         <v>5.16</v>
       </c>
       <c r="I22">
-        <f>ROUND(G22/F22,2)</f>
+        <f t="shared" si="1"/>
         <v>10.36</v>
       </c>
       <c r="J22">
@@ -8145,7 +8158,7 @@
         <v>51</v>
       </c>
       <c r="L22">
-        <f>IFERROR(ROUND(K22/J22,2),)</f>
+        <f t="shared" si="2"/>
         <v>4.25</v>
       </c>
       <c r="M22" t="s">
@@ -8181,11 +8194,11 @@
         <v>1204</v>
       </c>
       <c r="H23">
-        <f>ROUND(E23/D23,2)</f>
+        <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
       <c r="I23">
-        <f>ROUND(G23/F23,2)</f>
+        <f t="shared" si="1"/>
         <v>0.6</v>
       </c>
       <c r="J23">
@@ -8197,7 +8210,7 @@
         <v>0</v>
       </c>
       <c r="L23">
-        <f>IFERROR(ROUND(K23/J23,2),)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -8224,11 +8237,11 @@
         <v>218</v>
       </c>
       <c r="H24">
-        <f>ROUND(E24/D24,2)</f>
+        <f t="shared" si="0"/>
         <v>0.08</v>
       </c>
       <c r="I24">
-        <f>ROUND(G24/F24,2)</f>
+        <f t="shared" si="1"/>
         <v>0.56999999999999995</v>
       </c>
       <c r="J24">
@@ -8240,7 +8253,7 @@
         <v>0</v>
       </c>
       <c r="L24">
-        <f>IFERROR(ROUND(K24/J24,2),)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -8267,11 +8280,11 @@
         <v>7</v>
       </c>
       <c r="H25">
-        <f>ROUND(E25/D25,2)</f>
+        <f t="shared" si="0"/>
         <v>0.03</v>
       </c>
       <c r="I25">
-        <f>ROUND(G25/F25,2)</f>
+        <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
       <c r="J25">
@@ -8283,7 +8296,7 @@
         <v>0</v>
       </c>
       <c r="L25">
-        <f>IFERROR(ROUND(K25/J25,2),)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -8310,11 +8323,11 @@
         <v>941</v>
       </c>
       <c r="H26">
-        <f>ROUND(E26/D26,2)</f>
+        <f t="shared" si="0"/>
         <v>2.11</v>
       </c>
       <c r="I26">
-        <f>ROUND(G26/F26,2)</f>
+        <f t="shared" si="1"/>
         <v>6.23</v>
       </c>
       <c r="J26">
@@ -8326,7 +8339,7 @@
         <v>0</v>
       </c>
       <c r="L26">
-        <f>IFERROR(ROUND(K26/J26,2),)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M26" t="s">
@@ -8362,11 +8375,11 @@
         <v>73</v>
       </c>
       <c r="H27">
-        <f>ROUND(E27/D27,2)</f>
+        <f t="shared" si="0"/>
         <v>0.37</v>
       </c>
       <c r="I27">
-        <f>ROUND(G27/F27,2)</f>
+        <f t="shared" si="1"/>
         <v>1.2</v>
       </c>
       <c r="J27">
@@ -8378,7 +8391,7 @@
         <v>0</v>
       </c>
       <c r="L27">
-        <f>IFERROR(ROUND(K27/J27,2),)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -8405,11 +8418,11 @@
         <v>809</v>
       </c>
       <c r="H28">
-        <f>ROUND(E28/D28,2)</f>
+        <f t="shared" si="0"/>
         <v>0.54</v>
       </c>
       <c r="I28">
-        <f>ROUND(G28/F28,2)</f>
+        <f t="shared" si="1"/>
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="J28">
@@ -8421,7 +8434,7 @@
         <v>0</v>
       </c>
       <c r="L28">
-        <f>IFERROR(ROUND(K28/J28,2),)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -8448,11 +8461,11 @@
         <v>284</v>
       </c>
       <c r="H29">
-        <f>ROUND(E29/D29,2)</f>
+        <f t="shared" si="0"/>
         <v>7.33</v>
       </c>
       <c r="I29">
-        <f>ROUND(G29/F29,2)</f>
+        <f t="shared" si="1"/>
         <v>2.33</v>
       </c>
       <c r="J29">
@@ -8464,7 +8477,7 @@
         <v>0</v>
       </c>
       <c r="L29">
-        <f>IFERROR(ROUND(K29/J29,2),)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -8491,11 +8504,11 @@
         <v>665</v>
       </c>
       <c r="H30">
-        <f>ROUND(E30/D30,2)</f>
+        <f t="shared" si="0"/>
         <v>0.9</v>
       </c>
       <c r="I30">
-        <f>ROUND(G30/F30,2)</f>
+        <f t="shared" si="1"/>
         <v>1.92</v>
       </c>
       <c r="J30">
@@ -8507,7 +8520,7 @@
         <v>0</v>
       </c>
       <c r="L30">
-        <f>IFERROR(ROUND(K30/J30,2),)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -8534,11 +8547,11 @@
         <v>144</v>
       </c>
       <c r="H31">
-        <f>ROUND(E31/D31,2)</f>
+        <f t="shared" si="0"/>
         <v>2.33</v>
       </c>
       <c r="I31">
-        <f>ROUND(G31/F31,2)</f>
+        <f t="shared" si="1"/>
         <v>0.78</v>
       </c>
       <c r="J31">
@@ -8550,7 +8563,7 @@
         <v>0</v>
       </c>
       <c r="L31">
-        <f>IFERROR(ROUND(K31/J31,2),)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -8577,19 +8590,2149 @@
         <v>240</v>
       </c>
       <c r="H32">
+        <f t="shared" si="0"/>
+        <v>0.35</v>
+      </c>
+      <c r="I32">
+        <f t="shared" si="1"/>
+        <v>0.4</v>
+      </c>
+      <c r="J32">
+        <f>F32-IFERROR(VLOOKUP($A32,'0703'!$A$1:G81,6,FALSE),IFERROR(VLOOKUP($C32,'0703'!$C$1:G81,4,FALSE),F32-D32))</f>
+        <v>7</v>
+      </c>
+      <c r="K32">
+        <f>G32-IFERROR(VLOOKUP($A32,'0703'!$A$1:H81,7,FALSE),IFERROR(VLOOKUP($C32,'0703'!$C$1:H81,5,FALSE),G32-E32))</f>
+        <v>0</v>
+      </c>
+      <c r="L32">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>79</v>
+      </c>
+      <c r="B33" t="s">
+        <v>11</v>
+      </c>
+      <c r="C33" s="1">
+        <v>46153</v>
+      </c>
+      <c r="D33">
+        <v>6</v>
+      </c>
+      <c r="E33">
+        <v>5</v>
+      </c>
+      <c r="F33">
+        <v>134</v>
+      </c>
+      <c r="G33">
+        <v>98</v>
+      </c>
+      <c r="H33">
+        <f t="shared" si="0"/>
+        <v>0.83</v>
+      </c>
+      <c r="I33">
+        <f t="shared" si="1"/>
+        <v>0.73</v>
+      </c>
+      <c r="J33">
+        <f>F33-IFERROR(VLOOKUP($A33,'0703'!$A$1:G82,6,FALSE),IFERROR(VLOOKUP($C33,'0703'!$C$1:G82,4,FALSE),F33-D33))</f>
+        <v>0</v>
+      </c>
+      <c r="K33">
+        <f>G33-IFERROR(VLOOKUP($A33,'0703'!$A$1:H82,7,FALSE),IFERROR(VLOOKUP($C33,'0703'!$C$1:H82,5,FALSE),G33-E33))</f>
+        <v>0</v>
+      </c>
+      <c r="L33">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34" t="s">
+        <v>11</v>
+      </c>
+      <c r="C34" s="1">
+        <v>46129</v>
+      </c>
+      <c r="D34">
+        <v>13</v>
+      </c>
+      <c r="E34">
+        <v>12</v>
+      </c>
+      <c r="F34">
+        <v>403</v>
+      </c>
+      <c r="G34">
+        <v>129</v>
+      </c>
+      <c r="H34">
+        <f t="shared" si="0"/>
+        <v>0.92</v>
+      </c>
+      <c r="I34">
+        <f t="shared" si="1"/>
+        <v>0.32</v>
+      </c>
+      <c r="J34">
+        <f>F34-IFERROR(VLOOKUP($A34,'0703'!$A$1:G83,6,FALSE),IFERROR(VLOOKUP($C34,'0703'!$C$1:G83,4,FALSE),F34-D34))</f>
+        <v>0</v>
+      </c>
+      <c r="K34">
+        <f>G34-IFERROR(VLOOKUP($A34,'0703'!$A$1:H83,7,FALSE),IFERROR(VLOOKUP($C34,'0703'!$C$1:H83,5,FALSE),G34-E34))</f>
+        <v>0</v>
+      </c>
+      <c r="L34">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>87</v>
+      </c>
+      <c r="B35" t="s">
+        <v>11</v>
+      </c>
+      <c r="C35" s="1">
+        <v>46103</v>
+      </c>
+      <c r="D35">
+        <v>5</v>
+      </c>
+      <c r="E35">
+        <v>6</v>
+      </c>
+      <c r="F35">
+        <v>192</v>
+      </c>
+      <c r="G35">
+        <v>115</v>
+      </c>
+      <c r="H35">
+        <f t="shared" si="0"/>
+        <v>1.2</v>
+      </c>
+      <c r="I35">
+        <f t="shared" si="1"/>
+        <v>0.6</v>
+      </c>
+      <c r="J35">
+        <f>F35-IFERROR(VLOOKUP($A35,'0703'!$A$1:G84,6,FALSE),IFERROR(VLOOKUP($C35,'0703'!$C$1:G84,4,FALSE),F35-D35))</f>
+        <v>0</v>
+      </c>
+      <c r="K35">
+        <f>G35-IFERROR(VLOOKUP($A35,'0703'!$A$1:H84,7,FALSE),IFERROR(VLOOKUP($C35,'0703'!$C$1:H84,5,FALSE),G35-E35))</f>
+        <v>0</v>
+      </c>
+      <c r="L35">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>56</v>
+      </c>
+      <c r="B36" t="s">
+        <v>11</v>
+      </c>
+      <c r="C36" s="1">
+        <v>46063</v>
+      </c>
+      <c r="D36">
+        <v>1</v>
+      </c>
+      <c r="E36">
+        <v>9</v>
+      </c>
+      <c r="F36">
+        <v>248</v>
+      </c>
+      <c r="G36">
+        <v>523</v>
+      </c>
+      <c r="H36">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+      <c r="I36">
+        <f t="shared" si="1"/>
+        <v>2.11</v>
+      </c>
+      <c r="J36">
+        <f>F36-IFERROR(VLOOKUP($A36,'0703'!$A$1:G85,6,FALSE),IFERROR(VLOOKUP($C36,'0703'!$C$1:G85,4,FALSE),F36-D36))</f>
+        <v>0</v>
+      </c>
+      <c r="K36">
+        <f>G36-IFERROR(VLOOKUP($A36,'0703'!$A$1:H85,7,FALSE),IFERROR(VLOOKUP($C36,'0703'!$C$1:H85,5,FALSE),G36-E36))</f>
+        <v>0</v>
+      </c>
+      <c r="L36">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37" t="s">
+        <v>11</v>
+      </c>
+      <c r="C37" s="1">
+        <v>46031</v>
+      </c>
+      <c r="D37">
+        <v>183</v>
+      </c>
+      <c r="E37">
+        <v>9</v>
+      </c>
+      <c r="F37">
+        <v>3042</v>
+      </c>
+      <c r="G37">
+        <v>1465</v>
+      </c>
+      <c r="H37">
+        <f t="shared" si="0"/>
+        <v>0.05</v>
+      </c>
+      <c r="I37">
+        <f t="shared" si="1"/>
+        <v>0.48</v>
+      </c>
+      <c r="J37">
+        <f>F37-IFERROR(VLOOKUP($A37,'0703'!$A$1:G86,6,FALSE),IFERROR(VLOOKUP($C37,'0703'!$C$1:G86,4,FALSE),F37-D37))</f>
+        <v>4</v>
+      </c>
+      <c r="K37">
+        <f>G37-IFERROR(VLOOKUP($A37,'0703'!$A$1:H86,7,FALSE),IFERROR(VLOOKUP($C37,'0703'!$C$1:H86,5,FALSE),G37-E37))</f>
+        <v>0</v>
+      </c>
+      <c r="L37">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>80</v>
+      </c>
+      <c r="B38" t="s">
+        <v>11</v>
+      </c>
+      <c r="C38" s="1">
+        <v>45995</v>
+      </c>
+      <c r="D38">
+        <v>11</v>
+      </c>
+      <c r="E38">
+        <v>7</v>
+      </c>
+      <c r="F38">
+        <v>4483</v>
+      </c>
+      <c r="G38">
+        <v>1457</v>
+      </c>
+      <c r="H38">
+        <f t="shared" si="0"/>
+        <v>0.64</v>
+      </c>
+      <c r="I38">
+        <f t="shared" si="1"/>
+        <v>0.33</v>
+      </c>
+      <c r="J38">
+        <f>F38-IFERROR(VLOOKUP($A38,'0703'!$A$1:G87,6,FALSE),IFERROR(VLOOKUP($C38,'0703'!$C$1:G87,4,FALSE),F38-D38))</f>
+        <v>0</v>
+      </c>
+      <c r="K38">
+        <f>G38-IFERROR(VLOOKUP($A38,'0703'!$A$1:H87,7,FALSE),IFERROR(VLOOKUP($C38,'0703'!$C$1:H87,5,FALSE),G38-E38))</f>
+        <v>0</v>
+      </c>
+      <c r="L38">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>88</v>
+      </c>
+      <c r="B39" t="s">
+        <v>11</v>
+      </c>
+      <c r="C39" s="1">
+        <v>45990</v>
+      </c>
+      <c r="D39">
+        <v>27</v>
+      </c>
+      <c r="E39">
+        <v>1</v>
+      </c>
+      <c r="F39">
+        <v>1106</v>
+      </c>
+      <c r="G39">
+        <v>1170</v>
+      </c>
+      <c r="H39">
+        <f t="shared" si="0"/>
+        <v>0.04</v>
+      </c>
+      <c r="I39">
+        <f t="shared" si="1"/>
+        <v>1.06</v>
+      </c>
+      <c r="J39">
+        <f>F39-IFERROR(VLOOKUP($A39,'0703'!$A$1:G88,6,FALSE),IFERROR(VLOOKUP($C39,'0703'!$C$1:G88,4,FALSE),F39-D39))</f>
+        <v>10</v>
+      </c>
+      <c r="K39">
+        <f>G39-IFERROR(VLOOKUP($A39,'0703'!$A$1:H88,7,FALSE),IFERROR(VLOOKUP($C39,'0703'!$C$1:H88,5,FALSE),G39-E39))</f>
+        <v>0</v>
+      </c>
+      <c r="L39">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>61</v>
+      </c>
+      <c r="B40" t="s">
+        <v>11</v>
+      </c>
+      <c r="C40" s="1">
+        <v>45982</v>
+      </c>
+      <c r="D40">
+        <v>33</v>
+      </c>
+      <c r="E40">
+        <v>3</v>
+      </c>
+      <c r="F40">
+        <v>340</v>
+      </c>
+      <c r="G40">
+        <v>940</v>
+      </c>
+      <c r="H40">
+        <f t="shared" si="0"/>
+        <v>0.09</v>
+      </c>
+      <c r="I40">
+        <f t="shared" si="1"/>
+        <v>2.76</v>
+      </c>
+      <c r="J40">
+        <f>F40-IFERROR(VLOOKUP($A40,'0703'!$A$1:G89,6,FALSE),IFERROR(VLOOKUP($C40,'0703'!$C$1:G89,4,FALSE),F40-D40))</f>
+        <v>0</v>
+      </c>
+      <c r="K40">
+        <f>G40-IFERROR(VLOOKUP($A40,'0703'!$A$1:H89,7,FALSE),IFERROR(VLOOKUP($C40,'0703'!$C$1:H89,5,FALSE),G40-E40))</f>
+        <v>0</v>
+      </c>
+      <c r="L40">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>62</v>
+      </c>
+      <c r="B41" t="s">
+        <v>11</v>
+      </c>
+      <c r="C41" s="1">
+        <v>45973</v>
+      </c>
+      <c r="D41">
+        <v>14</v>
+      </c>
+      <c r="E41">
+        <v>3</v>
+      </c>
+      <c r="F41">
+        <v>20300</v>
+      </c>
+      <c r="G41">
+        <v>6787</v>
+      </c>
+      <c r="H41">
+        <f t="shared" si="0"/>
+        <v>0.21</v>
+      </c>
+      <c r="I41">
+        <f t="shared" si="1"/>
+        <v>0.33</v>
+      </c>
+      <c r="J41">
+        <f>F41-IFERROR(VLOOKUP($A41,'0703'!$A$1:G90,6,FALSE),IFERROR(VLOOKUP($C41,'0703'!$C$1:G90,4,FALSE),F41-D41))</f>
+        <v>1</v>
+      </c>
+      <c r="K41">
+        <f>G41-IFERROR(VLOOKUP($A41,'0703'!$A$1:H90,7,FALSE),IFERROR(VLOOKUP($C41,'0703'!$C$1:H90,5,FALSE),G41-E41))</f>
+        <v>0</v>
+      </c>
+      <c r="L41">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>64</v>
+      </c>
+      <c r="B42" t="s">
+        <v>11</v>
+      </c>
+      <c r="C42" s="1">
+        <v>45937</v>
+      </c>
+      <c r="D42">
+        <v>19</v>
+      </c>
+      <c r="E42">
+        <v>5</v>
+      </c>
+      <c r="F42">
+        <v>994</v>
+      </c>
+      <c r="G42">
+        <v>654</v>
+      </c>
+      <c r="H42">
+        <f t="shared" si="0"/>
+        <v>0.26</v>
+      </c>
+      <c r="I42">
+        <f t="shared" si="1"/>
+        <v>0.66</v>
+      </c>
+      <c r="J42">
+        <f>F42-IFERROR(VLOOKUP($A42,'0703'!$A$1:G91,6,FALSE),IFERROR(VLOOKUP($C42,'0703'!$C$1:G91,4,FALSE),F42-D42))</f>
+        <v>0</v>
+      </c>
+      <c r="K42">
+        <f>G42-IFERROR(VLOOKUP($A42,'0703'!$A$1:H91,7,FALSE),IFERROR(VLOOKUP($C42,'0703'!$C$1:H91,5,FALSE),G42-E42))</f>
+        <v>0</v>
+      </c>
+      <c r="L42">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>65</v>
+      </c>
+      <c r="B43" t="s">
+        <v>11</v>
+      </c>
+      <c r="C43" s="1">
+        <v>45933</v>
+      </c>
+      <c r="D43">
+        <v>23</v>
+      </c>
+      <c r="E43">
+        <v>1</v>
+      </c>
+      <c r="F43">
+        <v>356</v>
+      </c>
+      <c r="G43">
+        <v>539</v>
+      </c>
+      <c r="H43">
+        <f t="shared" si="0"/>
+        <v>0.04</v>
+      </c>
+      <c r="I43">
+        <f t="shared" si="1"/>
+        <v>1.51</v>
+      </c>
+      <c r="J43">
+        <f>F43-IFERROR(VLOOKUP($A43,'0703'!$A$1:G92,6,FALSE),IFERROR(VLOOKUP($C43,'0703'!$C$1:G92,4,FALSE),F43-D43))</f>
+        <v>0</v>
+      </c>
+      <c r="K43">
+        <f>G43-IFERROR(VLOOKUP($A43,'0703'!$A$1:H92,7,FALSE),IFERROR(VLOOKUP($C43,'0703'!$C$1:H92,5,FALSE),G43-E43))</f>
+        <v>0</v>
+      </c>
+      <c r="L43">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>66</v>
+      </c>
+      <c r="B44" t="s">
+        <v>11</v>
+      </c>
+      <c r="C44" s="1">
+        <v>45930</v>
+      </c>
+      <c r="D44">
+        <v>13</v>
+      </c>
+      <c r="E44">
+        <v>2</v>
+      </c>
+      <c r="F44">
+        <v>409</v>
+      </c>
+      <c r="G44">
+        <v>314</v>
+      </c>
+      <c r="H44">
+        <f t="shared" si="0"/>
+        <v>0.15</v>
+      </c>
+      <c r="I44">
+        <f t="shared" si="1"/>
+        <v>0.77</v>
+      </c>
+      <c r="J44">
+        <f>F44-IFERROR(VLOOKUP($A44,'0703'!$A$1:G93,6,FALSE),IFERROR(VLOOKUP($C44,'0703'!$C$1:G93,4,FALSE),F44-D44))</f>
+        <v>0</v>
+      </c>
+      <c r="K44">
+        <f>G44-IFERROR(VLOOKUP($A44,'0703'!$A$1:H93,7,FALSE),IFERROR(VLOOKUP($C44,'0703'!$C$1:H93,5,FALSE),G44-E44))</f>
+        <v>0</v>
+      </c>
+      <c r="L44">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>67</v>
+      </c>
+      <c r="B45" t="s">
+        <v>11</v>
+      </c>
+      <c r="C45" s="1">
+        <v>45927</v>
+      </c>
+      <c r="D45">
+        <v>3</v>
+      </c>
+      <c r="E45">
+        <v>1</v>
+      </c>
+      <c r="F45">
+        <v>239</v>
+      </c>
+      <c r="G45">
+        <v>680</v>
+      </c>
+      <c r="H45">
+        <f t="shared" si="0"/>
+        <v>0.33</v>
+      </c>
+      <c r="I45">
+        <f t="shared" si="1"/>
+        <v>2.85</v>
+      </c>
+      <c r="J45">
+        <f>F45-IFERROR(VLOOKUP($A45,'0703'!$A$1:G94,6,FALSE),IFERROR(VLOOKUP($C45,'0703'!$C$1:G94,4,FALSE),F45-D45))</f>
+        <v>0</v>
+      </c>
+      <c r="K45">
+        <f>G45-IFERROR(VLOOKUP($A45,'0703'!$A$1:H94,7,FALSE),IFERROR(VLOOKUP($C45,'0703'!$C$1:H94,5,FALSE),G45-E45))</f>
+        <v>0</v>
+      </c>
+      <c r="L45">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>89</v>
+      </c>
+      <c r="B46" t="s">
+        <v>11</v>
+      </c>
+      <c r="C46" s="1">
+        <v>45921</v>
+      </c>
+      <c r="D46">
+        <v>1</v>
+      </c>
+      <c r="E46">
+        <v>1</v>
+      </c>
+      <c r="F46">
+        <v>567</v>
+      </c>
+      <c r="G46">
+        <v>1011</v>
+      </c>
+      <c r="H46">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="I46">
+        <f t="shared" si="1"/>
+        <v>1.78</v>
+      </c>
+      <c r="J46">
+        <f>F46-IFERROR(VLOOKUP($A46,'0703'!$A$1:G95,6,FALSE),IFERROR(VLOOKUP($C46,'0703'!$C$1:G95,4,FALSE),F46-D46))</f>
+        <v>0</v>
+      </c>
+      <c r="K46">
+        <f>G46-IFERROR(VLOOKUP($A46,'0703'!$A$1:H95,7,FALSE),IFERROR(VLOOKUP($C46,'0703'!$C$1:H95,5,FALSE),G46-E46))</f>
+        <v>0</v>
+      </c>
+      <c r="L46">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>98</v>
+      </c>
+      <c r="B47" t="s">
+        <v>11</v>
+      </c>
+      <c r="C47" s="1">
+        <v>45911</v>
+      </c>
+      <c r="D47">
+        <v>8</v>
+      </c>
+      <c r="E47">
+        <v>1</v>
+      </c>
+      <c r="F47">
+        <v>384</v>
+      </c>
+      <c r="G47">
+        <v>391</v>
+      </c>
+      <c r="H47">
+        <f t="shared" si="0"/>
+        <v>0.13</v>
+      </c>
+      <c r="I47">
+        <f t="shared" si="1"/>
+        <v>1.02</v>
+      </c>
+      <c r="J47">
+        <f>F47-IFERROR(VLOOKUP($A47,'0703'!$A$1:G96,6,FALSE),IFERROR(VLOOKUP($C47,'0703'!$C$1:G96,4,FALSE),F47-D47))</f>
+        <v>8</v>
+      </c>
+      <c r="K47">
+        <f>G47-IFERROR(VLOOKUP($A47,'0703'!$A$1:H96,7,FALSE),IFERROR(VLOOKUP($C47,'0703'!$C$1:H96,5,FALSE),G47-E47))</f>
+        <v>1</v>
+      </c>
+      <c r="L47">
+        <f t="shared" si="2"/>
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>68</v>
+      </c>
+      <c r="B48" t="s">
+        <v>11</v>
+      </c>
+      <c r="C48" s="1">
+        <v>45899</v>
+      </c>
+      <c r="D48">
+        <v>4</v>
+      </c>
+      <c r="E48">
+        <v>1</v>
+      </c>
+      <c r="F48">
+        <v>805</v>
+      </c>
+      <c r="G48">
+        <v>538</v>
+      </c>
+      <c r="H48">
+        <f t="shared" si="0"/>
+        <v>0.25</v>
+      </c>
+      <c r="I48">
+        <f t="shared" si="1"/>
+        <v>0.67</v>
+      </c>
+      <c r="J48">
+        <f>F48-IFERROR(VLOOKUP($A48,'0703'!$A$1:G97,6,FALSE),IFERROR(VLOOKUP($C48,'0703'!$C$1:G97,4,FALSE),F48-D48))</f>
+        <v>0</v>
+      </c>
+      <c r="K48">
+        <f>G48-IFERROR(VLOOKUP($A48,'0703'!$A$1:H97,7,FALSE),IFERROR(VLOOKUP($C48,'0703'!$C$1:H97,5,FALSE),G48-E48))</f>
+        <v>0</v>
+      </c>
+      <c r="L48">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="10:11" x14ac:dyDescent="0.25">
+      <c r="J49" t="s">
+        <v>99</v>
+      </c>
+      <c r="K49">
+        <f>ROUND(SUM(K2:K48),2)</f>
+        <v>578</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2009A2F-80FA-46B5-8206-45390004EEE8}">
+  <dimension ref="A1:O47"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>90</v>
+      </c>
+      <c r="I1" t="s">
+        <v>91</v>
+      </c>
+      <c r="J1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K1" t="s">
+        <v>93</v>
+      </c>
+      <c r="L1" t="s">
+        <v>100</v>
+      </c>
+      <c r="M1" t="s">
+        <v>95</v>
+      </c>
+      <c r="N1" t="s">
+        <v>96</v>
+      </c>
+      <c r="O1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="1">
+        <v>46207</v>
+      </c>
+      <c r="D2">
+        <v>211</v>
+      </c>
+      <c r="E2">
+        <v>166</v>
+      </c>
+      <c r="F2">
+        <v>211</v>
+      </c>
+      <c r="G2">
+        <v>166</v>
+      </c>
+      <c r="H2">
+        <f>ROUND(E2/D2,2)</f>
+        <v>0.79</v>
+      </c>
+      <c r="I2">
+        <f>ROUND(G2/F2,2)</f>
+        <v>0.79</v>
+      </c>
+      <c r="J2">
+        <f>F2-IFERROR(VLOOKUP($A2,'0704'!$A$1:G49,6,FALSE),IFERROR(VLOOKUP($C2,'0704'!$C$1:G49,4,FALSE),F2-D2))</f>
+        <v>211</v>
+      </c>
+      <c r="K2">
+        <f>G2-IFERROR(VLOOKUP($A2,'0704'!$A$1:H49,7,FALSE),IFERROR(VLOOKUP($C2,'0704'!$C$1:H49,5,FALSE),G2-E2))</f>
+        <v>166</v>
+      </c>
+      <c r="L2">
+        <f>IFERROR(ROUND(K2/J2,2),)</f>
+        <v>0.79</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>102</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="1">
+        <v>46207</v>
+      </c>
+      <c r="D3">
+        <v>54</v>
+      </c>
+      <c r="E3">
+        <v>509</v>
+      </c>
+      <c r="F3">
+        <v>54</v>
+      </c>
+      <c r="G3">
+        <v>509</v>
+      </c>
+      <c r="H3">
+        <f>ROUND(E3/D3,2)</f>
+        <v>9.43</v>
+      </c>
+      <c r="I3">
+        <f>ROUND(G3/F3,2)</f>
+        <v>9.43</v>
+      </c>
+      <c r="J3">
+        <f>F3-IFERROR(VLOOKUP($A3,'0704'!$A$1:G50,6,FALSE),IFERROR(VLOOKUP($C3,'0704'!$C$1:G50,4,FALSE),F3-D3))</f>
+        <v>54</v>
+      </c>
+      <c r="K3">
+        <f>G3-IFERROR(VLOOKUP($A3,'0704'!$A$1:H50,7,FALSE),IFERROR(VLOOKUP($C3,'0704'!$C$1:H50,5,FALSE),G3-E3))</f>
+        <v>509</v>
+      </c>
+      <c r="L3">
+        <f>IFERROR(ROUND(K3/J3,2),)</f>
+        <v>9.43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="1">
+        <v>46205</v>
+      </c>
+      <c r="D4">
+        <v>2280</v>
+      </c>
+      <c r="E4">
+        <v>212</v>
+      </c>
+      <c r="F4">
+        <v>2280</v>
+      </c>
+      <c r="G4">
+        <v>212</v>
+      </c>
+      <c r="H4">
+        <f>ROUND(E4/D4,2)</f>
+        <v>0.09</v>
+      </c>
+      <c r="I4">
+        <f>ROUND(G4/F4,2)</f>
+        <v>0.09</v>
+      </c>
+      <c r="J4">
+        <f>F4-IFERROR(VLOOKUP($A4,'0704'!$A$1:G51,6,FALSE),IFERROR(VLOOKUP($C4,'0704'!$C$1:G51,4,FALSE),F4-D4))</f>
+        <v>98</v>
+      </c>
+      <c r="K4">
+        <f>G4-IFERROR(VLOOKUP($A4,'0704'!$A$1:H51,7,FALSE),IFERROR(VLOOKUP($C4,'0704'!$C$1:H51,5,FALSE),G4-E4))</f>
+        <v>37</v>
+      </c>
+      <c r="L4">
+        <f>IFERROR(ROUND(K4/J4,2),)</f>
+        <v>0.38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>82</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="1">
+        <v>46205</v>
+      </c>
+      <c r="D5">
+        <v>671</v>
+      </c>
+      <c r="E5">
+        <v>1129</v>
+      </c>
+      <c r="F5">
+        <v>671</v>
+      </c>
+      <c r="G5">
+        <v>1129</v>
+      </c>
+      <c r="H5">
+        <f>ROUND(E5/D5,2)</f>
+        <v>1.68</v>
+      </c>
+      <c r="I5">
+        <f>ROUND(G5/F5,2)</f>
+        <v>1.68</v>
+      </c>
+      <c r="J5">
+        <f>F5-IFERROR(VLOOKUP($A5,'0704'!$A$1:G52,6,FALSE),IFERROR(VLOOKUP($C5,'0704'!$C$1:G52,4,FALSE),F5-D5))</f>
+        <v>151</v>
+      </c>
+      <c r="K5">
+        <f>G5-IFERROR(VLOOKUP($A5,'0704'!$A$1:H52,7,FALSE),IFERROR(VLOOKUP($C5,'0704'!$C$1:H52,5,FALSE),G5-E5))</f>
+        <v>138</v>
+      </c>
+      <c r="L5">
+        <f>IFERROR(ROUND(K5/J5,2),)</f>
+        <v>0.91</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>75</v>
+      </c>
+      <c r="B6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="1">
+        <v>46204</v>
+      </c>
+      <c r="D6">
+        <v>588</v>
+      </c>
+      <c r="E6">
+        <v>255</v>
+      </c>
+      <c r="F6">
+        <v>588</v>
+      </c>
+      <c r="G6">
+        <v>255</v>
+      </c>
+      <c r="H6">
+        <f>ROUND(E6/D6,2)</f>
+        <v>0.43</v>
+      </c>
+      <c r="I6">
+        <f>ROUND(G6/F6,2)</f>
+        <v>0.43</v>
+      </c>
+      <c r="J6">
+        <f>F6-IFERROR(VLOOKUP($A6,'0704'!$A$1:G53,6,FALSE),IFERROR(VLOOKUP($C6,'0704'!$C$1:G53,4,FALSE),F6-D6))</f>
+        <v>56</v>
+      </c>
+      <c r="K6">
+        <f>G6-IFERROR(VLOOKUP($A6,'0704'!$A$1:H53,7,FALSE),IFERROR(VLOOKUP($C6,'0704'!$C$1:H53,5,FALSE),G6-E6))</f>
+        <v>14</v>
+      </c>
+      <c r="L6">
+        <f>IFERROR(ROUND(K6/J6,2),)</f>
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>76</v>
+      </c>
+      <c r="B7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="1">
+        <v>46204</v>
+      </c>
+      <c r="D7">
+        <v>159</v>
+      </c>
+      <c r="E7">
+        <v>332</v>
+      </c>
+      <c r="F7">
+        <v>159</v>
+      </c>
+      <c r="G7">
+        <v>332</v>
+      </c>
+      <c r="H7">
+        <f>ROUND(E7/D7,2)</f>
+        <v>2.09</v>
+      </c>
+      <c r="I7">
+        <f>ROUND(G7/F7,2)</f>
+        <v>2.09</v>
+      </c>
+      <c r="J7">
+        <f>F7-IFERROR(VLOOKUP($A7,'0704'!$A$1:G54,6,FALSE),IFERROR(VLOOKUP($C7,'0704'!$C$1:G54,4,FALSE),F7-D7))</f>
+        <v>10</v>
+      </c>
+      <c r="K7">
+        <f>G7-IFERROR(VLOOKUP($A7,'0704'!$A$1:H54,7,FALSE),IFERROR(VLOOKUP($C7,'0704'!$C$1:H54,5,FALSE),G7-E7))</f>
+        <v>15</v>
+      </c>
+      <c r="L7">
+        <f>IFERROR(ROUND(K7/J7,2),)</f>
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="1">
+        <v>46203</v>
+      </c>
+      <c r="D8">
+        <v>89</v>
+      </c>
+      <c r="E8">
+        <v>689</v>
+      </c>
+      <c r="F8">
+        <v>89</v>
+      </c>
+      <c r="G8">
+        <v>689</v>
+      </c>
+      <c r="H8">
+        <f>ROUND(E8/D8,2)</f>
+        <v>7.74</v>
+      </c>
+      <c r="I8">
+        <f>ROUND(G8/F8,2)</f>
+        <v>7.74</v>
+      </c>
+      <c r="J8">
+        <f>F8-IFERROR(VLOOKUP($A8,'0704'!$A$1:G55,6,FALSE),IFERROR(VLOOKUP($C8,'0704'!$C$1:G55,4,FALSE),F8-D8))</f>
+        <v>9</v>
+      </c>
+      <c r="K8">
+        <f>G8-IFERROR(VLOOKUP($A8,'0704'!$A$1:H55,7,FALSE),IFERROR(VLOOKUP($C8,'0704'!$C$1:H55,5,FALSE),G8-E8))</f>
+        <v>34</v>
+      </c>
+      <c r="L8">
+        <f>IFERROR(ROUND(K8/J8,2),)</f>
+        <v>3.78</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="1">
+        <v>46203</v>
+      </c>
+      <c r="D9">
+        <v>873</v>
+      </c>
+      <c r="E9">
+        <v>114</v>
+      </c>
+      <c r="F9">
+        <v>873</v>
+      </c>
+      <c r="G9">
+        <v>114</v>
+      </c>
+      <c r="H9">
+        <f>ROUND(E9/D9,2)</f>
+        <v>0.13</v>
+      </c>
+      <c r="I9">
+        <f>ROUND(G9/F9,2)</f>
+        <v>0.13</v>
+      </c>
+      <c r="J9">
+        <f>F9-IFERROR(VLOOKUP($A9,'0704'!$A$1:G56,6,FALSE),IFERROR(VLOOKUP($C9,'0704'!$C$1:G56,4,FALSE),F9-D9))</f>
+        <v>47</v>
+      </c>
+      <c r="K9">
+        <f>G9-IFERROR(VLOOKUP($A9,'0704'!$A$1:H56,7,FALSE),IFERROR(VLOOKUP($C9,'0704'!$C$1:H56,5,FALSE),G9-E9))</f>
+        <v>0</v>
+      </c>
+      <c r="L9">
+        <f>IFERROR(ROUND(K9/J9,2),)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" s="1">
+        <v>46202</v>
+      </c>
+      <c r="D10">
+        <v>108</v>
+      </c>
+      <c r="E10">
+        <v>1004</v>
+      </c>
+      <c r="F10">
+        <v>108</v>
+      </c>
+      <c r="G10">
+        <v>1004</v>
+      </c>
+      <c r="H10">
+        <f>ROUND(E10/D10,2)</f>
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="I10">
+        <f>ROUND(G10/F10,2)</f>
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="J10">
+        <f>F10-IFERROR(VLOOKUP($A10,'0704'!$A$1:G57,6,FALSE),IFERROR(VLOOKUP($C10,'0704'!$C$1:G57,4,FALSE),F10-D10))</f>
+        <v>4</v>
+      </c>
+      <c r="K10">
+        <f>G10-IFERROR(VLOOKUP($A10,'0704'!$A$1:H57,7,FALSE),IFERROR(VLOOKUP($C10,'0704'!$C$1:H57,5,FALSE),G10-E10))</f>
+        <v>86</v>
+      </c>
+      <c r="L10">
+        <f>IFERROR(ROUND(K10/J10,2),)</f>
+        <v>21.5</v>
+      </c>
+      <c r="M10" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" s="1">
+        <v>46202</v>
+      </c>
+      <c r="D11">
+        <v>514</v>
+      </c>
+      <c r="E11">
+        <v>205</v>
+      </c>
+      <c r="F11">
+        <v>514</v>
+      </c>
+      <c r="G11">
+        <v>205</v>
+      </c>
+      <c r="H11">
+        <f>ROUND(E11/D11,2)</f>
+        <v>0.4</v>
+      </c>
+      <c r="I11">
+        <f>ROUND(G11/F11,2)</f>
+        <v>0.4</v>
+      </c>
+      <c r="J11">
+        <f>F11-IFERROR(VLOOKUP($A11,'0704'!$A$1:G58,6,FALSE),IFERROR(VLOOKUP($C11,'0704'!$C$1:G58,4,FALSE),F11-D11))</f>
+        <v>12</v>
+      </c>
+      <c r="K11">
+        <f>G11-IFERROR(VLOOKUP($A11,'0704'!$A$1:H58,7,FALSE),IFERROR(VLOOKUP($C11,'0704'!$C$1:H58,5,FALSE),G11-E11))</f>
+        <v>0</v>
+      </c>
+      <c r="L11">
+        <f>IFERROR(ROUND(K11/J11,2),)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" s="1">
+        <v>46201</v>
+      </c>
+      <c r="D12">
+        <v>442</v>
+      </c>
+      <c r="E12">
+        <v>310</v>
+      </c>
+      <c r="F12">
+        <v>442</v>
+      </c>
+      <c r="G12">
+        <v>310</v>
+      </c>
+      <c r="H12">
+        <f>ROUND(E12/D12,2)</f>
+        <v>0.7</v>
+      </c>
+      <c r="I12">
+        <f>ROUND(G12/F12,2)</f>
+        <v>0.7</v>
+      </c>
+      <c r="J12">
+        <f>F12-IFERROR(VLOOKUP($A12,'0704'!$A$1:G59,6,FALSE),IFERROR(VLOOKUP($C12,'0704'!$C$1:G59,4,FALSE),F12-D12))</f>
+        <v>16</v>
+      </c>
+      <c r="K12">
+        <f>G12-IFERROR(VLOOKUP($A12,'0704'!$A$1:H59,7,FALSE),IFERROR(VLOOKUP($C12,'0704'!$C$1:H59,5,FALSE),G12-E12))</f>
+        <v>0</v>
+      </c>
+      <c r="L12">
+        <f>IFERROR(ROUND(K12/J12,2),)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C13" s="1">
+        <v>46201</v>
+      </c>
+      <c r="D13">
+        <v>328</v>
+      </c>
+      <c r="E13">
+        <v>967</v>
+      </c>
+      <c r="F13">
+        <v>328</v>
+      </c>
+      <c r="G13">
+        <v>967</v>
+      </c>
+      <c r="H13">
+        <f>ROUND(E13/D13,2)</f>
+        <v>2.95</v>
+      </c>
+      <c r="I13">
+        <f>ROUND(G13/F13,2)</f>
+        <v>2.95</v>
+      </c>
+      <c r="J13">
+        <f>F13-IFERROR(VLOOKUP($A13,'0704'!$A$1:G60,6,FALSE),IFERROR(VLOOKUP($C13,'0704'!$C$1:G60,4,FALSE),F13-D13))</f>
+        <v>5</v>
+      </c>
+      <c r="K13">
+        <f>G13-IFERROR(VLOOKUP($A13,'0704'!$A$1:H60,7,FALSE),IFERROR(VLOOKUP($C13,'0704'!$C$1:H60,5,FALSE),G13-E13))</f>
+        <v>0</v>
+      </c>
+      <c r="L13">
+        <f>IFERROR(ROUND(K13/J13,2),)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" t="s">
+        <v>11</v>
+      </c>
+      <c r="C14" s="1">
+        <v>46200</v>
+      </c>
+      <c r="D14">
+        <v>154</v>
+      </c>
+      <c r="E14">
+        <v>437</v>
+      </c>
+      <c r="F14">
+        <v>168</v>
+      </c>
+      <c r="G14">
+        <v>549</v>
+      </c>
+      <c r="H14">
+        <f>ROUND(E14/D14,2)</f>
+        <v>2.84</v>
+      </c>
+      <c r="I14">
+        <f>ROUND(G14/F14,2)</f>
+        <v>3.27</v>
+      </c>
+      <c r="J14">
+        <f>F14-IFERROR(VLOOKUP($A14,'0704'!$A$1:G61,6,FALSE),IFERROR(VLOOKUP($C14,'0704'!$C$1:G61,4,FALSE),F14-D14))</f>
+        <v>9</v>
+      </c>
+      <c r="K14">
+        <f>G14-IFERROR(VLOOKUP($A14,'0704'!$A$1:H61,7,FALSE),IFERROR(VLOOKUP($C14,'0704'!$C$1:H61,5,FALSE),G14-E14))</f>
+        <v>6</v>
+      </c>
+      <c r="L14">
+        <f>IFERROR(ROUND(K14/J14,2),)</f>
+        <v>0.67</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>19</v>
+      </c>
+      <c r="B15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C15" s="1">
+        <v>46199</v>
+      </c>
+      <c r="D15">
+        <v>44</v>
+      </c>
+      <c r="E15">
+        <v>114</v>
+      </c>
+      <c r="F15">
+        <v>121</v>
+      </c>
+      <c r="G15">
+        <v>430</v>
+      </c>
+      <c r="H15">
+        <f>ROUND(E15/D15,2)</f>
+        <v>2.59</v>
+      </c>
+      <c r="I15">
+        <f>ROUND(G15/F15,2)</f>
+        <v>3.55</v>
+      </c>
+      <c r="J15">
+        <f>F15-IFERROR(VLOOKUP($A15,'0704'!$A$1:G62,6,FALSE),IFERROR(VLOOKUP($C15,'0704'!$C$1:G62,4,FALSE),F15-D15))</f>
+        <v>1</v>
+      </c>
+      <c r="K15">
+        <f>G15-IFERROR(VLOOKUP($A15,'0704'!$A$1:H62,7,FALSE),IFERROR(VLOOKUP($C15,'0704'!$C$1:H62,5,FALSE),G15-E15))</f>
+        <v>0</v>
+      </c>
+      <c r="L15">
+        <f>IFERROR(ROUND(K15/J15,2),)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16" t="s">
+        <v>11</v>
+      </c>
+      <c r="C16" s="1">
+        <v>46198</v>
+      </c>
+      <c r="D16">
+        <v>86</v>
+      </c>
+      <c r="E16">
+        <v>352</v>
+      </c>
+      <c r="F16">
+        <v>215</v>
+      </c>
+      <c r="G16">
+        <v>1454</v>
+      </c>
+      <c r="H16">
+        <f>ROUND(E16/D16,2)</f>
+        <v>4.09</v>
+      </c>
+      <c r="I16">
+        <f>ROUND(G16/F16,2)</f>
+        <v>6.76</v>
+      </c>
+      <c r="J16">
+        <f>F16-IFERROR(VLOOKUP($A16,'0704'!$A$1:G63,6,FALSE),IFERROR(VLOOKUP($C16,'0704'!$C$1:G63,4,FALSE),F16-D16))</f>
+        <v>7</v>
+      </c>
+      <c r="K16">
+        <f>G16-IFERROR(VLOOKUP($A16,'0704'!$A$1:H63,7,FALSE),IFERROR(VLOOKUP($C16,'0704'!$C$1:H63,5,FALSE),G16-E16))</f>
+        <v>17</v>
+      </c>
+      <c r="L16">
+        <f>IFERROR(ROUND(K16/J16,2),)</f>
+        <v>2.4300000000000002</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" s="1">
+        <v>46197</v>
+      </c>
+      <c r="D17">
+        <v>50</v>
+      </c>
+      <c r="E17">
+        <v>234</v>
+      </c>
+      <c r="F17">
+        <v>126</v>
+      </c>
+      <c r="G17">
+        <v>650</v>
+      </c>
+      <c r="H17">
+        <f>ROUND(E17/D17,2)</f>
+        <v>4.68</v>
+      </c>
+      <c r="I17">
+        <f>ROUND(G17/F17,2)</f>
+        <v>5.16</v>
+      </c>
+      <c r="J17">
+        <f>F17-IFERROR(VLOOKUP($A17,'0704'!$A$1:G64,6,FALSE),IFERROR(VLOOKUP($C17,'0704'!$C$1:G64,4,FALSE),F17-D17))</f>
+        <v>4</v>
+      </c>
+      <c r="K17">
+        <f>G17-IFERROR(VLOOKUP($A17,'0704'!$A$1:H64,7,FALSE),IFERROR(VLOOKUP($C17,'0704'!$C$1:H64,5,FALSE),G17-E17))</f>
+        <v>0</v>
+      </c>
+      <c r="L17">
+        <f>IFERROR(ROUND(K17/J17,2),)</f>
+        <v>0</v>
+      </c>
+      <c r="M17" t="s">
+        <v>23</v>
+      </c>
+      <c r="N17" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>24</v>
+      </c>
+      <c r="B18" t="s">
+        <v>13</v>
+      </c>
+      <c r="C18" s="1">
+        <v>46196</v>
+      </c>
+      <c r="D18">
+        <v>72</v>
+      </c>
+      <c r="E18">
+        <v>10</v>
+      </c>
+      <c r="F18">
+        <v>932</v>
+      </c>
+      <c r="G18">
+        <v>281</v>
+      </c>
+      <c r="H18">
+        <f>ROUND(E18/D18,2)</f>
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="I18">
+        <f>ROUND(G18/F18,2)</f>
+        <v>0.3</v>
+      </c>
+      <c r="J18">
+        <f>F18-IFERROR(VLOOKUP($A18,'0704'!$A$1:G65,6,FALSE),IFERROR(VLOOKUP($C18,'0704'!$C$1:G65,4,FALSE),F18-D18))</f>
+        <v>10</v>
+      </c>
+      <c r="K18">
+        <f>G18-IFERROR(VLOOKUP($A18,'0704'!$A$1:H65,7,FALSE),IFERROR(VLOOKUP($C18,'0704'!$C$1:H65,5,FALSE),G18-E18))</f>
+        <v>0</v>
+      </c>
+      <c r="L18">
+        <f>IFERROR(ROUND(K18/J18,2),)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>25</v>
+      </c>
+      <c r="B19" t="s">
+        <v>11</v>
+      </c>
+      <c r="C19" s="1">
+        <v>46196</v>
+      </c>
+      <c r="D19">
+        <v>61</v>
+      </c>
+      <c r="E19">
+        <v>279</v>
+      </c>
+      <c r="F19">
+        <v>199</v>
+      </c>
+      <c r="G19">
+        <v>1399</v>
+      </c>
+      <c r="H19">
+        <f>ROUND(E19/D19,2)</f>
+        <v>4.57</v>
+      </c>
+      <c r="I19">
+        <f>ROUND(G19/F19,2)</f>
+        <v>7.03</v>
+      </c>
+      <c r="J19">
+        <f>F19-IFERROR(VLOOKUP($A19,'0704'!$A$1:G66,6,FALSE),IFERROR(VLOOKUP($C19,'0704'!$C$1:G66,4,FALSE),F19-D19))</f>
+        <v>4</v>
+      </c>
+      <c r="K19">
+        <f>G19-IFERROR(VLOOKUP($A19,'0704'!$A$1:H66,7,FALSE),IFERROR(VLOOKUP($C19,'0704'!$C$1:H66,5,FALSE),G19-E19))</f>
+        <v>34</v>
+      </c>
+      <c r="L19">
+        <f>IFERROR(ROUND(K19/J19,2),)</f>
+        <v>8.5</v>
+      </c>
+      <c r="M19" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" t="s">
+        <v>11</v>
+      </c>
+      <c r="C20" s="1">
+        <v>46195</v>
+      </c>
+      <c r="D20">
+        <v>62</v>
+      </c>
+      <c r="E20">
+        <v>329</v>
+      </c>
+      <c r="F20">
+        <v>152</v>
+      </c>
+      <c r="G20">
+        <v>730</v>
+      </c>
+      <c r="H20">
+        <f>ROUND(E20/D20,2)</f>
+        <v>5.31</v>
+      </c>
+      <c r="I20">
+        <f>ROUND(G20/F20,2)</f>
+        <v>4.8</v>
+      </c>
+      <c r="J20">
+        <f>F20-IFERROR(VLOOKUP($A20,'0704'!$A$1:G67,6,FALSE),IFERROR(VLOOKUP($C20,'0704'!$C$1:G67,4,FALSE),F20-D20))</f>
+        <v>0</v>
+      </c>
+      <c r="K20">
+        <f>G20-IFERROR(VLOOKUP($A20,'0704'!$A$1:H67,7,FALSE),IFERROR(VLOOKUP($C20,'0704'!$C$1:H67,5,FALSE),G20-E20))</f>
+        <v>0</v>
+      </c>
+      <c r="L20">
+        <f>IFERROR(ROUND(K20/J20,2),)</f>
+        <v>0</v>
+      </c>
+      <c r="M20" t="s">
+        <v>27</v>
+      </c>
+      <c r="N20" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" t="s">
+        <v>11</v>
+      </c>
+      <c r="C21" s="1">
+        <v>46194</v>
+      </c>
+      <c r="D21">
+        <v>13</v>
+      </c>
+      <c r="E21">
+        <v>95</v>
+      </c>
+      <c r="F21">
+        <v>154</v>
+      </c>
+      <c r="G21">
+        <v>1024</v>
+      </c>
+      <c r="H21">
+        <f>ROUND(E21/D21,2)</f>
+        <v>7.31</v>
+      </c>
+      <c r="I21">
+        <f>ROUND(G21/F21,2)</f>
+        <v>6.65</v>
+      </c>
+      <c r="J21">
+        <f>F21-IFERROR(VLOOKUP($A21,'0704'!$A$1:G68,6,FALSE),IFERROR(VLOOKUP($C21,'0704'!$C$1:G68,4,FALSE),F21-D21))</f>
+        <v>0</v>
+      </c>
+      <c r="K21">
+        <f>G21-IFERROR(VLOOKUP($A21,'0704'!$A$1:H68,7,FALSE),IFERROR(VLOOKUP($C21,'0704'!$C$1:H68,5,FALSE),G21-E21))</f>
+        <v>0</v>
+      </c>
+      <c r="L21">
+        <f>IFERROR(ROUND(K21/J21,2),)</f>
+        <v>0</v>
+      </c>
+      <c r="M21" t="s">
+        <v>29</v>
+      </c>
+      <c r="N21" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>31</v>
+      </c>
+      <c r="B22" t="s">
+        <v>32</v>
+      </c>
+      <c r="C22" s="1">
+        <v>46193</v>
+      </c>
+      <c r="D22">
+        <v>17</v>
+      </c>
+      <c r="E22">
+        <v>5</v>
+      </c>
+      <c r="F22">
+        <v>149</v>
+      </c>
+      <c r="G22">
+        <v>114</v>
+      </c>
+      <c r="H22">
+        <f>ROUND(E22/D22,2)</f>
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="I22">
+        <f>ROUND(G22/F22,2)</f>
+        <v>0.77</v>
+      </c>
+      <c r="J22">
+        <f>F22-IFERROR(VLOOKUP($A22,'0704'!$A$1:G69,6,FALSE),IFERROR(VLOOKUP($C22,'0704'!$C$1:G69,4,FALSE),F22-D22))</f>
+        <v>1</v>
+      </c>
+      <c r="K22">
+        <f>G22-IFERROR(VLOOKUP($A22,'0704'!$A$1:H69,7,FALSE),IFERROR(VLOOKUP($C22,'0704'!$C$1:H69,5,FALSE),G22-E22))</f>
+        <v>0</v>
+      </c>
+      <c r="L22">
+        <f>IFERROR(ROUND(K22/J22,2),)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>33</v>
+      </c>
+      <c r="B23" t="s">
+        <v>11</v>
+      </c>
+      <c r="C23" s="1">
+        <v>46193</v>
+      </c>
+      <c r="D23">
+        <v>51</v>
+      </c>
+      <c r="E23">
+        <v>89</v>
+      </c>
+      <c r="F23">
+        <v>184</v>
+      </c>
+      <c r="G23">
+        <v>1668</v>
+      </c>
+      <c r="H23">
+        <f>ROUND(E23/D23,2)</f>
+        <v>1.75</v>
+      </c>
+      <c r="I23">
+        <f>ROUND(G23/F23,2)</f>
+        <v>9.07</v>
+      </c>
+      <c r="J23">
+        <f>F23-IFERROR(VLOOKUP($A23,'0704'!$A$1:G70,6,FALSE),IFERROR(VLOOKUP($C23,'0704'!$C$1:G70,4,FALSE),F23-D23))</f>
+        <v>23</v>
+      </c>
+      <c r="K23">
+        <f>G23-IFERROR(VLOOKUP($A23,'0704'!$A$1:H70,7,FALSE),IFERROR(VLOOKUP($C23,'0704'!$C$1:H70,5,FALSE),G23-E23))</f>
+        <v>0</v>
+      </c>
+      <c r="L23">
+        <f>IFERROR(ROUND(K23/J23,2),)</f>
+        <v>0</v>
+      </c>
+      <c r="M23" t="s">
+        <v>34</v>
+      </c>
+      <c r="N23" t="s">
+        <v>35</v>
+      </c>
+      <c r="O23" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>36</v>
+      </c>
+      <c r="B24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C24" s="1">
+        <v>46192</v>
+      </c>
+      <c r="D24">
+        <v>118</v>
+      </c>
+      <c r="E24">
+        <v>38</v>
+      </c>
+      <c r="F24">
+        <v>2015</v>
+      </c>
+      <c r="G24">
+        <v>1204</v>
+      </c>
+      <c r="H24">
+        <f>ROUND(E24/D24,2)</f>
+        <v>0.32</v>
+      </c>
+      <c r="I24">
+        <f>ROUND(G24/F24,2)</f>
+        <v>0.6</v>
+      </c>
+      <c r="J24">
+        <f>F24-IFERROR(VLOOKUP($A24,'0704'!$A$1:G71,6,FALSE),IFERROR(VLOOKUP($C24,'0704'!$C$1:G71,4,FALSE),F24-D24))</f>
+        <v>2</v>
+      </c>
+      <c r="K24">
+        <f>G24-IFERROR(VLOOKUP($A24,'0704'!$A$1:H71,7,FALSE),IFERROR(VLOOKUP($C24,'0704'!$C$1:H71,5,FALSE),G24-E24))</f>
+        <v>0</v>
+      </c>
+      <c r="L24">
+        <f>IFERROR(ROUND(K24/J24,2),)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>37</v>
+      </c>
+      <c r="B25" t="s">
+        <v>11</v>
+      </c>
+      <c r="C25" s="1">
+        <v>46191</v>
+      </c>
+      <c r="D25">
+        <v>76</v>
+      </c>
+      <c r="E25">
+        <v>7</v>
+      </c>
+      <c r="F25">
+        <v>390</v>
+      </c>
+      <c r="G25">
+        <v>218</v>
+      </c>
+      <c r="H25">
+        <f>ROUND(E25/D25,2)</f>
+        <v>0.09</v>
+      </c>
+      <c r="I25">
+        <f>ROUND(G25/F25,2)</f>
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="J25">
+        <f>F25-IFERROR(VLOOKUP($A25,'0704'!$A$1:G72,6,FALSE),IFERROR(VLOOKUP($C25,'0704'!$C$1:G72,4,FALSE),F25-D25))</f>
+        <v>5</v>
+      </c>
+      <c r="K25">
+        <f>G25-IFERROR(VLOOKUP($A25,'0704'!$A$1:H72,7,FALSE),IFERROR(VLOOKUP($C25,'0704'!$C$1:H72,5,FALSE),G25-E25))</f>
+        <v>0</v>
+      </c>
+      <c r="L25">
+        <f>IFERROR(ROUND(K25/J25,2),)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>38</v>
+      </c>
+      <c r="B26" t="s">
+        <v>11</v>
+      </c>
+      <c r="C26" s="1">
+        <v>46190</v>
+      </c>
+      <c r="D26">
+        <v>30</v>
+      </c>
+      <c r="E26">
+        <v>1</v>
+      </c>
+      <c r="F26">
+        <v>701</v>
+      </c>
+      <c r="G26">
+        <v>7</v>
+      </c>
+      <c r="H26">
+        <f>ROUND(E26/D26,2)</f>
+        <v>0.03</v>
+      </c>
+      <c r="I26">
+        <f>ROUND(G26/F26,2)</f>
+        <v>0.01</v>
+      </c>
+      <c r="J26">
+        <f>F26-IFERROR(VLOOKUP($A26,'0704'!$A$1:G73,6,FALSE),IFERROR(VLOOKUP($C26,'0704'!$C$1:G73,4,FALSE),F26-D26))</f>
+        <v>1</v>
+      </c>
+      <c r="K26">
+        <f>G26-IFERROR(VLOOKUP($A26,'0704'!$A$1:H73,7,FALSE),IFERROR(VLOOKUP($C26,'0704'!$C$1:H73,5,FALSE),G26-E26))</f>
+        <v>0</v>
+      </c>
+      <c r="L26">
+        <f>IFERROR(ROUND(K26/J26,2),)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>39</v>
+      </c>
+      <c r="B27" t="s">
+        <v>11</v>
+      </c>
+      <c r="C27" s="1">
+        <v>46189</v>
+      </c>
+      <c r="D27">
+        <v>15</v>
+      </c>
+      <c r="E27">
+        <v>19</v>
+      </c>
+      <c r="F27">
+        <v>157</v>
+      </c>
+      <c r="G27">
+        <v>941</v>
+      </c>
+      <c r="H27">
+        <f>ROUND(E27/D27,2)</f>
+        <v>1.27</v>
+      </c>
+      <c r="I27">
+        <f>ROUND(G27/F27,2)</f>
+        <v>5.99</v>
+      </c>
+      <c r="J27">
+        <f>F27-IFERROR(VLOOKUP($A27,'0704'!$A$1:G74,6,FALSE),IFERROR(VLOOKUP($C27,'0704'!$C$1:G74,4,FALSE),F27-D27))</f>
+        <v>6</v>
+      </c>
+      <c r="K27">
+        <f>G27-IFERROR(VLOOKUP($A27,'0704'!$A$1:H74,7,FALSE),IFERROR(VLOOKUP($C27,'0704'!$C$1:H74,5,FALSE),G27-E27))</f>
+        <v>0</v>
+      </c>
+      <c r="L27">
+        <f>IFERROR(ROUND(K27/J27,2),)</f>
+        <v>0</v>
+      </c>
+      <c r="M27" t="s">
+        <v>40</v>
+      </c>
+      <c r="N27" t="s">
+        <v>41</v>
+      </c>
+      <c r="O27" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>86</v>
+      </c>
+      <c r="B28" t="s">
+        <v>11</v>
+      </c>
+      <c r="C28" s="1">
+        <v>46188</v>
+      </c>
+      <c r="D28">
+        <v>20</v>
+      </c>
+      <c r="E28">
+        <v>7</v>
+      </c>
+      <c r="F28">
+        <v>62</v>
+      </c>
+      <c r="G28">
+        <v>73</v>
+      </c>
+      <c r="H28">
+        <f>ROUND(E28/D28,2)</f>
+        <v>0.35</v>
+      </c>
+      <c r="I28">
+        <f>ROUND(G28/F28,2)</f>
+        <v>1.18</v>
+      </c>
+      <c r="J28">
+        <f>F28-IFERROR(VLOOKUP($A28,'0704'!$A$1:G75,6,FALSE),IFERROR(VLOOKUP($C28,'0704'!$C$1:G75,4,FALSE),F28-D28))</f>
+        <v>1</v>
+      </c>
+      <c r="K28">
+        <f>G28-IFERROR(VLOOKUP($A28,'0704'!$A$1:H75,7,FALSE),IFERROR(VLOOKUP($C28,'0704'!$C$1:H75,5,FALSE),G28-E28))</f>
+        <v>0</v>
+      </c>
+      <c r="L28">
+        <f>IFERROR(ROUND(K28/J28,2),)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>43</v>
+      </c>
+      <c r="B29" t="s">
+        <v>11</v>
+      </c>
+      <c r="C29" s="1">
+        <v>46187</v>
+      </c>
+      <c r="D29">
+        <v>203</v>
+      </c>
+      <c r="E29">
+        <v>132</v>
+      </c>
+      <c r="F29">
+        <v>11112</v>
+      </c>
+      <c r="G29">
+        <v>834</v>
+      </c>
+      <c r="H29">
+        <f>ROUND(E29/D29,2)</f>
+        <v>0.65</v>
+      </c>
+      <c r="I29">
+        <f>ROUND(G29/F29,2)</f>
+        <v>0.08</v>
+      </c>
+      <c r="J29">
+        <f>F29-IFERROR(VLOOKUP($A29,'0704'!$A$1:G76,6,FALSE),IFERROR(VLOOKUP($C29,'0704'!$C$1:G76,4,FALSE),F29-D29))</f>
+        <v>16</v>
+      </c>
+      <c r="K29">
+        <f>G29-IFERROR(VLOOKUP($A29,'0704'!$A$1:H76,7,FALSE),IFERROR(VLOOKUP($C29,'0704'!$C$1:H76,5,FALSE),G29-E29))</f>
+        <v>25</v>
+      </c>
+      <c r="L29">
+        <f>IFERROR(ROUND(K29/J29,2),)</f>
+        <v>1.56</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>47</v>
+      </c>
+      <c r="B30" t="s">
+        <v>11</v>
+      </c>
+      <c r="C30" s="1">
+        <v>46182</v>
+      </c>
+      <c r="D30">
+        <v>3</v>
+      </c>
+      <c r="E30">
+        <v>22</v>
+      </c>
+      <c r="F30">
+        <v>122</v>
+      </c>
+      <c r="G30">
+        <v>284</v>
+      </c>
+      <c r="H30">
+        <f>ROUND(E30/D30,2)</f>
+        <v>7.33</v>
+      </c>
+      <c r="I30">
+        <f>ROUND(G30/F30,2)</f>
+        <v>2.33</v>
+      </c>
+      <c r="J30">
+        <f>F30-IFERROR(VLOOKUP($A30,'0704'!$A$1:G77,6,FALSE),IFERROR(VLOOKUP($C30,'0704'!$C$1:G77,4,FALSE),F30-D30))</f>
+        <v>0</v>
+      </c>
+      <c r="K30">
+        <f>G30-IFERROR(VLOOKUP($A30,'0704'!$A$1:H77,7,FALSE),IFERROR(VLOOKUP($C30,'0704'!$C$1:H77,5,FALSE),G30-E30))</f>
+        <v>0</v>
+      </c>
+      <c r="L30">
+        <f>IFERROR(ROUND(K30/J30,2),)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>48</v>
+      </c>
+      <c r="B31" t="s">
+        <v>11</v>
+      </c>
+      <c r="C31" s="1">
+        <v>46177</v>
+      </c>
+      <c r="D31">
+        <v>16</v>
+      </c>
+      <c r="E31">
+        <v>19</v>
+      </c>
+      <c r="F31">
+        <v>346</v>
+      </c>
+      <c r="G31">
+        <v>665</v>
+      </c>
+      <c r="H31">
+        <f>ROUND(E31/D31,2)</f>
+        <v>1.19</v>
+      </c>
+      <c r="I31">
+        <f>ROUND(G31/F31,2)</f>
+        <v>1.92</v>
+      </c>
+      <c r="J31">
+        <f>F31-IFERROR(VLOOKUP($A31,'0704'!$A$1:G78,6,FALSE),IFERROR(VLOOKUP($C31,'0704'!$C$1:G78,4,FALSE),F31-D31))</f>
+        <v>0</v>
+      </c>
+      <c r="K31">
+        <f>G31-IFERROR(VLOOKUP($A31,'0704'!$A$1:H78,7,FALSE),IFERROR(VLOOKUP($C31,'0704'!$C$1:H78,5,FALSE),G31-E31))</f>
+        <v>0</v>
+      </c>
+      <c r="L31">
+        <f>IFERROR(ROUND(K31/J31,2),)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>52</v>
+      </c>
+      <c r="B32" t="s">
+        <v>11</v>
+      </c>
+      <c r="C32" s="1">
+        <v>46164</v>
+      </c>
+      <c r="D32">
+        <v>35</v>
+      </c>
+      <c r="E32">
+        <v>6</v>
+      </c>
+      <c r="F32">
+        <v>597</v>
+      </c>
+      <c r="G32">
+        <v>240</v>
+      </c>
+      <c r="H32">
         <f>ROUND(E32/D32,2)</f>
-        <v>0.35</v>
+        <v>0.17</v>
       </c>
       <c r="I32">
         <f>ROUND(G32/F32,2)</f>
         <v>0.4</v>
       </c>
       <c r="J32">
-        <f>F32-IFERROR(VLOOKUP($A32,'0703'!$A$1:G81,6,FALSE),IFERROR(VLOOKUP($C32,'0703'!$C$1:G81,4,FALSE),F32-D32))</f>
-        <v>7</v>
+        <f>F32-IFERROR(VLOOKUP($A32,'0704'!$A$1:G79,6,FALSE),IFERROR(VLOOKUP($C32,'0704'!$C$1:G79,4,FALSE),F32-D32))</f>
+        <v>1</v>
       </c>
       <c r="K32">
-        <f>G32-IFERROR(VLOOKUP($A32,'0703'!$A$1:H81,7,FALSE),IFERROR(VLOOKUP($C32,'0703'!$C$1:H81,5,FALSE),G32-E32))</f>
+        <f>G32-IFERROR(VLOOKUP($A32,'0704'!$A$1:H79,7,FALSE),IFERROR(VLOOKUP($C32,'0704'!$C$1:H79,5,FALSE),G32-E32))</f>
         <v>0</v>
       </c>
       <c r="L32">
@@ -8628,11 +10771,11 @@
         <v>0.73</v>
       </c>
       <c r="J33">
-        <f>F33-IFERROR(VLOOKUP($A33,'0703'!$A$1:G82,6,FALSE),IFERROR(VLOOKUP($C33,'0703'!$C$1:G82,4,FALSE),F33-D33))</f>
+        <f>F33-IFERROR(VLOOKUP($A33,'0704'!$A$1:G80,6,FALSE),IFERROR(VLOOKUP($C33,'0704'!$C$1:G80,4,FALSE),F33-D33))</f>
         <v>0</v>
       </c>
       <c r="K33">
-        <f>G33-IFERROR(VLOOKUP($A33,'0703'!$A$1:H82,7,FALSE),IFERROR(VLOOKUP($C33,'0703'!$C$1:H82,5,FALSE),G33-E33))</f>
+        <f>G33-IFERROR(VLOOKUP($A33,'0704'!$A$1:H80,7,FALSE),IFERROR(VLOOKUP($C33,'0704'!$C$1:H80,5,FALSE),G33-E33))</f>
         <v>0</v>
       </c>
       <c r="L33">
@@ -8651,31 +10794,31 @@
         <v>46129</v>
       </c>
       <c r="D34">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E34">
         <v>12</v>
       </c>
       <c r="F34">
-        <v>403</v>
+        <v>407</v>
       </c>
       <c r="G34">
         <v>129</v>
       </c>
       <c r="H34">
         <f>ROUND(E34/D34,2)</f>
-        <v>0.92</v>
+        <v>0.75</v>
       </c>
       <c r="I34">
         <f>ROUND(G34/F34,2)</f>
         <v>0.32</v>
       </c>
       <c r="J34">
-        <f>F34-IFERROR(VLOOKUP($A34,'0703'!$A$1:G83,6,FALSE),IFERROR(VLOOKUP($C34,'0703'!$C$1:G83,4,FALSE),F34-D34))</f>
-        <v>0</v>
+        <f>F34-IFERROR(VLOOKUP($A34,'0704'!$A$1:G81,6,FALSE),IFERROR(VLOOKUP($C34,'0704'!$C$1:G81,4,FALSE),F34-D34))</f>
+        <v>4</v>
       </c>
       <c r="K34">
-        <f>G34-IFERROR(VLOOKUP($A34,'0703'!$A$1:H83,7,FALSE),IFERROR(VLOOKUP($C34,'0703'!$C$1:H83,5,FALSE),G34-E34))</f>
+        <f>G34-IFERROR(VLOOKUP($A34,'0704'!$A$1:H81,7,FALSE),IFERROR(VLOOKUP($C34,'0704'!$C$1:H81,5,FALSE),G34-E34))</f>
         <v>0</v>
       </c>
       <c r="L34">
@@ -8685,83 +10828,83 @@
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="B35" t="s">
         <v>11</v>
       </c>
       <c r="C35" s="1">
-        <v>46103</v>
+        <v>46113</v>
       </c>
       <c r="D35">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="E35">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F35">
-        <v>192</v>
+        <v>381</v>
       </c>
       <c r="G35">
-        <v>115</v>
+        <v>178</v>
       </c>
       <c r="H35">
         <f>ROUND(E35/D35,2)</f>
-        <v>1.2</v>
+        <v>0.19</v>
       </c>
       <c r="I35">
         <f>ROUND(G35/F35,2)</f>
-        <v>0.6</v>
+        <v>0.47</v>
       </c>
       <c r="J35">
-        <f>F35-IFERROR(VLOOKUP($A35,'0703'!$A$1:G84,6,FALSE),IFERROR(VLOOKUP($C35,'0703'!$C$1:G84,4,FALSE),F35-D35))</f>
-        <v>0</v>
+        <f>F35-IFERROR(VLOOKUP($A35,'0704'!$A$1:G82,6,FALSE),IFERROR(VLOOKUP($C35,'0704'!$C$1:G82,4,FALSE),F35-D35))</f>
+        <v>16</v>
       </c>
       <c r="K35">
-        <f>G35-IFERROR(VLOOKUP($A35,'0703'!$A$1:H84,7,FALSE),IFERROR(VLOOKUP($C35,'0703'!$C$1:H84,5,FALSE),G35-E35))</f>
-        <v>0</v>
+        <f>G35-IFERROR(VLOOKUP($A35,'0704'!$A$1:H82,7,FALSE),IFERROR(VLOOKUP($C35,'0704'!$C$1:H82,5,FALSE),G35-E35))</f>
+        <v>3</v>
       </c>
       <c r="L35">
         <f>IFERROR(ROUND(K35/J35,2),)</f>
-        <v>0</v>
+        <v>0.19</v>
       </c>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>56</v>
+        <v>87</v>
       </c>
       <c r="B36" t="s">
         <v>11</v>
       </c>
       <c r="C36" s="1">
-        <v>46063</v>
+        <v>46103</v>
       </c>
       <c r="D36">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E36">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="F36">
-        <v>248</v>
+        <v>192</v>
       </c>
       <c r="G36">
-        <v>523</v>
+        <v>115</v>
       </c>
       <c r="H36">
         <f>ROUND(E36/D36,2)</f>
-        <v>9</v>
+        <v>1.2</v>
       </c>
       <c r="I36">
         <f>ROUND(G36/F36,2)</f>
-        <v>2.11</v>
+        <v>0.6</v>
       </c>
       <c r="J36">
-        <f>F36-IFERROR(VLOOKUP($A36,'0703'!$A$1:G85,6,FALSE),IFERROR(VLOOKUP($C36,'0703'!$C$1:G85,4,FALSE),F36-D36))</f>
+        <f>F36-IFERROR(VLOOKUP($A36,'0704'!$A$1:G83,6,FALSE),IFERROR(VLOOKUP($C36,'0704'!$C$1:G83,4,FALSE),F36-D36))</f>
         <v>0</v>
       </c>
       <c r="K36">
-        <f>G36-IFERROR(VLOOKUP($A36,'0703'!$A$1:H85,7,FALSE),IFERROR(VLOOKUP($C36,'0703'!$C$1:H85,5,FALSE),G36-E36))</f>
+        <f>G36-IFERROR(VLOOKUP($A36,'0704'!$A$1:H83,7,FALSE),IFERROR(VLOOKUP($C36,'0704'!$C$1:H83,5,FALSE),G36-E36))</f>
         <v>0</v>
       </c>
       <c r="L36">
@@ -8771,40 +10914,40 @@
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B37" t="s">
         <v>11</v>
       </c>
       <c r="C37" s="1">
-        <v>46031</v>
+        <v>46063</v>
       </c>
       <c r="D37">
-        <v>183</v>
+        <v>2</v>
       </c>
       <c r="E37">
         <v>9</v>
       </c>
       <c r="F37">
-        <v>3042</v>
+        <v>249</v>
       </c>
       <c r="G37">
-        <v>1465</v>
+        <v>523</v>
       </c>
       <c r="H37">
         <f>ROUND(E37/D37,2)</f>
-        <v>0.05</v>
+        <v>4.5</v>
       </c>
       <c r="I37">
         <f>ROUND(G37/F37,2)</f>
-        <v>0.48</v>
+        <v>2.1</v>
       </c>
       <c r="J37">
-        <f>F37-IFERROR(VLOOKUP($A37,'0703'!$A$1:G86,6,FALSE),IFERROR(VLOOKUP($C37,'0703'!$C$1:G86,4,FALSE),F37-D37))</f>
-        <v>4</v>
+        <f>F37-IFERROR(VLOOKUP($A37,'0704'!$A$1:G84,6,FALSE),IFERROR(VLOOKUP($C37,'0704'!$C$1:G84,4,FALSE),F37-D37))</f>
+        <v>1</v>
       </c>
       <c r="K37">
-        <f>G37-IFERROR(VLOOKUP($A37,'0703'!$A$1:H86,7,FALSE),IFERROR(VLOOKUP($C37,'0703'!$C$1:H86,5,FALSE),G37-E37))</f>
+        <f>G37-IFERROR(VLOOKUP($A37,'0704'!$A$1:H84,7,FALSE),IFERROR(VLOOKUP($C37,'0704'!$C$1:H84,5,FALSE),G37-E37))</f>
         <v>0</v>
       </c>
       <c r="L37">
@@ -8823,31 +10966,31 @@
         <v>45995</v>
       </c>
       <c r="D38">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E38">
         <v>7</v>
       </c>
       <c r="F38">
-        <v>4483</v>
+        <v>4484</v>
       </c>
       <c r="G38">
         <v>1457</v>
       </c>
       <c r="H38">
         <f>ROUND(E38/D38,2)</f>
-        <v>0.64</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="I38">
         <f>ROUND(G38/F38,2)</f>
-        <v>0.33</v>
+        <v>0.32</v>
       </c>
       <c r="J38">
-        <f>F38-IFERROR(VLOOKUP($A38,'0703'!$A$1:G87,6,FALSE),IFERROR(VLOOKUP($C38,'0703'!$C$1:G87,4,FALSE),F38-D38))</f>
-        <v>0</v>
+        <f>F38-IFERROR(VLOOKUP($A38,'0704'!$A$1:G85,6,FALSE),IFERROR(VLOOKUP($C38,'0704'!$C$1:G85,4,FALSE),F38-D38))</f>
+        <v>1</v>
       </c>
       <c r="K38">
-        <f>G38-IFERROR(VLOOKUP($A38,'0703'!$A$1:H87,7,FALSE),IFERROR(VLOOKUP($C38,'0703'!$C$1:H87,5,FALSE),G38-E38))</f>
+        <f>G38-IFERROR(VLOOKUP($A38,'0704'!$A$1:H85,7,FALSE),IFERROR(VLOOKUP($C38,'0704'!$C$1:H85,5,FALSE),G38-E38))</f>
         <v>0</v>
       </c>
       <c r="L38">
@@ -8866,13 +11009,13 @@
         <v>45990</v>
       </c>
       <c r="D39">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E39">
         <v>1</v>
       </c>
       <c r="F39">
-        <v>1106</v>
+        <v>1107</v>
       </c>
       <c r="G39">
         <v>1170</v>
@@ -8886,11 +11029,11 @@
         <v>1.06</v>
       </c>
       <c r="J39">
-        <f>F39-IFERROR(VLOOKUP($A39,'0703'!$A$1:G88,6,FALSE),IFERROR(VLOOKUP($C39,'0703'!$C$1:G88,4,FALSE),F39-D39))</f>
-        <v>10</v>
+        <f>F39-IFERROR(VLOOKUP($A39,'0704'!$A$1:G86,6,FALSE),IFERROR(VLOOKUP($C39,'0704'!$C$1:G86,4,FALSE),F39-D39))</f>
+        <v>1</v>
       </c>
       <c r="K39">
-        <f>G39-IFERROR(VLOOKUP($A39,'0703'!$A$1:H88,7,FALSE),IFERROR(VLOOKUP($C39,'0703'!$C$1:H88,5,FALSE),G39-E39))</f>
+        <f>G39-IFERROR(VLOOKUP($A39,'0704'!$A$1:H86,7,FALSE),IFERROR(VLOOKUP($C39,'0704'!$C$1:H86,5,FALSE),G39-E39))</f>
         <v>0</v>
       </c>
       <c r="L39">
@@ -8929,11 +11072,11 @@
         <v>2.76</v>
       </c>
       <c r="J40">
-        <f>F40-IFERROR(VLOOKUP($A40,'0703'!$A$1:G89,6,FALSE),IFERROR(VLOOKUP($C40,'0703'!$C$1:G89,4,FALSE),F40-D40))</f>
+        <f>F40-IFERROR(VLOOKUP($A40,'0704'!$A$1:G87,6,FALSE),IFERROR(VLOOKUP($C40,'0704'!$C$1:G87,4,FALSE),F40-D40))</f>
         <v>0</v>
       </c>
       <c r="K40">
-        <f>G40-IFERROR(VLOOKUP($A40,'0703'!$A$1:H89,7,FALSE),IFERROR(VLOOKUP($C40,'0703'!$C$1:H89,5,FALSE),G40-E40))</f>
+        <f>G40-IFERROR(VLOOKUP($A40,'0704'!$A$1:H87,7,FALSE),IFERROR(VLOOKUP($C40,'0704'!$C$1:H87,5,FALSE),G40-E40))</f>
         <v>0</v>
       </c>
       <c r="L40">
@@ -8952,31 +11095,31 @@
         <v>45973</v>
       </c>
       <c r="D41">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E41">
         <v>3</v>
       </c>
       <c r="F41">
-        <v>20300</v>
+        <v>20301</v>
       </c>
       <c r="G41">
         <v>6787</v>
       </c>
       <c r="H41">
         <f>ROUND(E41/D41,2)</f>
-        <v>0.21</v>
+        <v>0.27</v>
       </c>
       <c r="I41">
         <f>ROUND(G41/F41,2)</f>
         <v>0.33</v>
       </c>
       <c r="J41">
-        <f>F41-IFERROR(VLOOKUP($A41,'0703'!$A$1:G90,6,FALSE),IFERROR(VLOOKUP($C41,'0703'!$C$1:G90,4,FALSE),F41-D41))</f>
+        <f>F41-IFERROR(VLOOKUP($A41,'0704'!$A$1:G88,6,FALSE),IFERROR(VLOOKUP($C41,'0704'!$C$1:G88,4,FALSE),F41-D41))</f>
         <v>1</v>
       </c>
       <c r="K41">
-        <f>G41-IFERROR(VLOOKUP($A41,'0703'!$A$1:H90,7,FALSE),IFERROR(VLOOKUP($C41,'0703'!$C$1:H90,5,FALSE),G41-E41))</f>
+        <f>G41-IFERROR(VLOOKUP($A41,'0704'!$A$1:H88,7,FALSE),IFERROR(VLOOKUP($C41,'0704'!$C$1:H88,5,FALSE),G41-E41))</f>
         <v>0</v>
       </c>
       <c r="L41">
@@ -8986,40 +11129,40 @@
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B42" t="s">
         <v>11</v>
       </c>
       <c r="C42" s="1">
-        <v>45937</v>
+        <v>45933</v>
       </c>
       <c r="D42">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="E42">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F42">
-        <v>994</v>
+        <v>356</v>
       </c>
       <c r="G42">
-        <v>654</v>
-      </c>
-      <c r="H42">
+        <v>539</v>
+      </c>
+      <c r="H42" t="e">
         <f>ROUND(E42/D42,2)</f>
-        <v>0.26</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="I42">
         <f>ROUND(G42/F42,2)</f>
-        <v>0.66</v>
+        <v>1.51</v>
       </c>
       <c r="J42">
-        <f>F42-IFERROR(VLOOKUP($A42,'0703'!$A$1:G91,6,FALSE),IFERROR(VLOOKUP($C42,'0703'!$C$1:G91,4,FALSE),F42-D42))</f>
+        <f>F42-IFERROR(VLOOKUP($A42,'0704'!$A$1:G89,6,FALSE),IFERROR(VLOOKUP($C42,'0704'!$C$1:G89,4,FALSE),F42-D42))</f>
         <v>0</v>
       </c>
       <c r="K42">
-        <f>G42-IFERROR(VLOOKUP($A42,'0703'!$A$1:H91,7,FALSE),IFERROR(VLOOKUP($C42,'0703'!$C$1:H91,5,FALSE),G42-E42))</f>
+        <f>G42-IFERROR(VLOOKUP($A42,'0704'!$A$1:H89,7,FALSE),IFERROR(VLOOKUP($C42,'0704'!$C$1:H89,5,FALSE),G42-E42))</f>
         <v>0</v>
       </c>
       <c r="L42">
@@ -9029,40 +11172,40 @@
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B43" t="s">
         <v>11</v>
       </c>
       <c r="C43" s="1">
-        <v>45933</v>
+        <v>45930</v>
       </c>
       <c r="D43">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="E43">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F43">
-        <v>356</v>
+        <v>409</v>
       </c>
       <c r="G43">
-        <v>539</v>
+        <v>314</v>
       </c>
       <c r="H43">
         <f>ROUND(E43/D43,2)</f>
-        <v>0.04</v>
+        <v>0.15</v>
       </c>
       <c r="I43">
         <f>ROUND(G43/F43,2)</f>
-        <v>1.51</v>
+        <v>0.77</v>
       </c>
       <c r="J43">
-        <f>F43-IFERROR(VLOOKUP($A43,'0703'!$A$1:G92,6,FALSE),IFERROR(VLOOKUP($C43,'0703'!$C$1:G92,4,FALSE),F43-D43))</f>
+        <f>F43-IFERROR(VLOOKUP($A43,'0704'!$A$1:G90,6,FALSE),IFERROR(VLOOKUP($C43,'0704'!$C$1:G90,4,FALSE),F43-D43))</f>
         <v>0</v>
       </c>
       <c r="K43">
-        <f>G43-IFERROR(VLOOKUP($A43,'0703'!$A$1:H92,7,FALSE),IFERROR(VLOOKUP($C43,'0703'!$C$1:H92,5,FALSE),G43-E43))</f>
+        <f>G43-IFERROR(VLOOKUP($A43,'0704'!$A$1:H90,7,FALSE),IFERROR(VLOOKUP($C43,'0704'!$C$1:H90,5,FALSE),G43-E43))</f>
         <v>0</v>
       </c>
       <c r="L43">
@@ -9072,40 +11215,40 @@
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B44" t="s">
         <v>11</v>
       </c>
       <c r="C44" s="1">
-        <v>45930</v>
+        <v>45927</v>
       </c>
       <c r="D44">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="E44">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F44">
-        <v>409</v>
+        <v>239</v>
       </c>
       <c r="G44">
-        <v>314</v>
+        <v>680</v>
       </c>
       <c r="H44">
         <f>ROUND(E44/D44,2)</f>
-        <v>0.15</v>
+        <v>0.33</v>
       </c>
       <c r="I44">
         <f>ROUND(G44/F44,2)</f>
-        <v>0.77</v>
+        <v>2.85</v>
       </c>
       <c r="J44">
-        <f>F44-IFERROR(VLOOKUP($A44,'0703'!$A$1:G93,6,FALSE),IFERROR(VLOOKUP($C44,'0703'!$C$1:G93,4,FALSE),F44-D44))</f>
+        <f>F44-IFERROR(VLOOKUP($A44,'0704'!$A$1:G91,6,FALSE),IFERROR(VLOOKUP($C44,'0704'!$C$1:G91,4,FALSE),F44-D44))</f>
         <v>0</v>
       </c>
       <c r="K44">
-        <f>G44-IFERROR(VLOOKUP($A44,'0703'!$A$1:H93,7,FALSE),IFERROR(VLOOKUP($C44,'0703'!$C$1:H93,5,FALSE),G44-E44))</f>
+        <f>G44-IFERROR(VLOOKUP($A44,'0704'!$A$1:H91,7,FALSE),IFERROR(VLOOKUP($C44,'0704'!$C$1:H91,5,FALSE),G44-E44))</f>
         <v>0</v>
       </c>
       <c r="L44">
@@ -9115,40 +11258,40 @@
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>67</v>
+        <v>89</v>
       </c>
       <c r="B45" t="s">
         <v>11</v>
       </c>
       <c r="C45" s="1">
-        <v>45927</v>
+        <v>45921</v>
       </c>
       <c r="D45">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E45">
         <v>1</v>
       </c>
       <c r="F45">
-        <v>239</v>
+        <v>567</v>
       </c>
       <c r="G45">
-        <v>680</v>
+        <v>1011</v>
       </c>
       <c r="H45">
         <f>ROUND(E45/D45,2)</f>
-        <v>0.33</v>
+        <v>1</v>
       </c>
       <c r="I45">
         <f>ROUND(G45/F45,2)</f>
-        <v>2.85</v>
+        <v>1.78</v>
       </c>
       <c r="J45">
-        <f>F45-IFERROR(VLOOKUP($A45,'0703'!$A$1:G94,6,FALSE),IFERROR(VLOOKUP($C45,'0703'!$C$1:G94,4,FALSE),F45-D45))</f>
+        <f>F45-IFERROR(VLOOKUP($A45,'0704'!$A$1:G92,6,FALSE),IFERROR(VLOOKUP($C45,'0704'!$C$1:G92,4,FALSE),F45-D45))</f>
         <v>0</v>
       </c>
       <c r="K45">
-        <f>G45-IFERROR(VLOOKUP($A45,'0703'!$A$1:H94,7,FALSE),IFERROR(VLOOKUP($C45,'0703'!$C$1:H94,5,FALSE),G45-E45))</f>
+        <f>G45-IFERROR(VLOOKUP($A45,'0704'!$A$1:H92,7,FALSE),IFERROR(VLOOKUP($C45,'0704'!$C$1:H92,5,FALSE),G45-E45))</f>
         <v>0</v>
       </c>
       <c r="L45">
@@ -9158,40 +11301,40 @@
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="B46" t="s">
         <v>11</v>
       </c>
       <c r="C46" s="1">
-        <v>45921</v>
+        <v>45911</v>
       </c>
       <c r="D46">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E46">
         <v>1</v>
       </c>
       <c r="F46">
-        <v>567</v>
+        <v>386</v>
       </c>
       <c r="G46">
-        <v>1011</v>
+        <v>391</v>
       </c>
       <c r="H46">
         <f>ROUND(E46/D46,2)</f>
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="I46">
         <f>ROUND(G46/F46,2)</f>
-        <v>1.78</v>
+        <v>1.01</v>
       </c>
       <c r="J46">
-        <f>F46-IFERROR(VLOOKUP($A46,'0703'!$A$1:G95,6,FALSE),IFERROR(VLOOKUP($C46,'0703'!$C$1:G95,4,FALSE),F46-D46))</f>
-        <v>0</v>
+        <f>F46-IFERROR(VLOOKUP($A46,'0704'!$A$1:G93,6,FALSE),IFERROR(VLOOKUP($C46,'0704'!$C$1:G93,4,FALSE),F46-D46))</f>
+        <v>2</v>
       </c>
       <c r="K46">
-        <f>G46-IFERROR(VLOOKUP($A46,'0703'!$A$1:H95,7,FALSE),IFERROR(VLOOKUP($C46,'0703'!$C$1:H95,5,FALSE),G46-E46))</f>
+        <f>G46-IFERROR(VLOOKUP($A46,'0704'!$A$1:H93,7,FALSE),IFERROR(VLOOKUP($C46,'0704'!$C$1:H93,5,FALSE),G46-E46))</f>
         <v>0</v>
       </c>
       <c r="L46">
@@ -9200,98 +11343,12 @@
       </c>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>98</v>
-      </c>
-      <c r="B47" t="s">
-        <v>11</v>
-      </c>
-      <c r="C47" s="1">
-        <v>45911</v>
-      </c>
-      <c r="D47">
-        <v>8</v>
-      </c>
-      <c r="E47">
-        <v>1</v>
-      </c>
-      <c r="F47">
-        <v>384</v>
-      </c>
-      <c r="G47">
-        <v>391</v>
-      </c>
-      <c r="H47">
-        <f>ROUND(E47/D47,2)</f>
-        <v>0.13</v>
-      </c>
-      <c r="I47">
-        <f>ROUND(G47/F47,2)</f>
-        <v>1.02</v>
-      </c>
-      <c r="J47">
-        <f>F47-IFERROR(VLOOKUP($A47,'0703'!$A$1:G96,6,FALSE),IFERROR(VLOOKUP($C47,'0703'!$C$1:G96,4,FALSE),F47-D47))</f>
-        <v>8</v>
+      <c r="J47" t="s">
+        <v>99</v>
       </c>
       <c r="K47">
-        <f>G47-IFERROR(VLOOKUP($A47,'0703'!$A$1:H96,7,FALSE),IFERROR(VLOOKUP($C47,'0703'!$C$1:H96,5,FALSE),G47-E47))</f>
-        <v>1</v>
-      </c>
-      <c r="L47">
-        <f>IFERROR(ROUND(K47/J47,2),)</f>
-        <v>0.13</v>
-      </c>
-    </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>68</v>
-      </c>
-      <c r="B48" t="s">
-        <v>11</v>
-      </c>
-      <c r="C48" s="1">
-        <v>45899</v>
-      </c>
-      <c r="D48">
-        <v>4</v>
-      </c>
-      <c r="E48">
-        <v>1</v>
-      </c>
-      <c r="F48">
-        <v>805</v>
-      </c>
-      <c r="G48">
-        <v>538</v>
-      </c>
-      <c r="H48">
-        <f>ROUND(E48/D48,2)</f>
-        <v>0.25</v>
-      </c>
-      <c r="I48">
-        <f>ROUND(G48/F48,2)</f>
-        <v>0.67</v>
-      </c>
-      <c r="J48">
-        <f>F48-IFERROR(VLOOKUP($A48,'0703'!$A$1:G97,6,FALSE),IFERROR(VLOOKUP($C48,'0703'!$C$1:G97,4,FALSE),F48-D48))</f>
-        <v>0</v>
-      </c>
-      <c r="K48">
-        <f>G48-IFERROR(VLOOKUP($A48,'0703'!$A$1:H97,7,FALSE),IFERROR(VLOOKUP($C48,'0703'!$C$1:H97,5,FALSE),G48-E48))</f>
-        <v>0</v>
-      </c>
-      <c r="L48">
-        <f>IFERROR(ROUND(K48/J48,2),)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49" spans="10:11" x14ac:dyDescent="0.25">
-      <c r="J49" t="s">
-        <v>99</v>
-      </c>
-      <c r="K49">
-        <f>ROUND(SUM(K2:K48),2)</f>
-        <v>578</v>
+        <f>ROUND(SUM(K2:K46),2)</f>
+        <v>1084</v>
       </c>
     </row>
   </sheetData>

</xml_diff>